<commit_message>
Close 29 Apr 2026 open trade at model exit (-185 pts) and refresh analysis and report
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NXDNZiScC3GTCLADanc7h1
</commit_message>
<xml_diff>
--- a/analysis/ssr_live_vs_model_analysis.xlsx
+++ b/analysis/ssr_live_vs_model_analysis.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Hedge-era compare" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Deviation vs model" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Missed by period" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Hedge diagnostics" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Monthly" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Matched trades" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Model-only (missed)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Live-only" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Daily equity &amp; DD" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Data fixes" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hedge-era compare" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deviation vs model" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missed by period" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hedge diagnostics" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched trades" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model-only (missed)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live-only" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily equity &amp; DD" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data fixes" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -537,10 +537,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-9781.099999999999</v>
+        <v>-9926.599999999999</v>
       </c>
       <c r="C7" t="n">
-        <v>-10983.70817364118</v>
+        <v>-11129.20817364118</v>
       </c>
       <c r="D7" t="n">
         <v>-11309</v>
@@ -553,10 +553,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1043.8</v>
+        <v>898.3000000000003</v>
       </c>
       <c r="C8" t="n">
-        <v>576.5207263588188</v>
+        <v>431.0207263588188</v>
       </c>
       <c r="D8" t="n">
         <v>1088</v>
@@ -569,10 +569,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.9035741669669002</v>
+        <v>0.9170153996803663</v>
       </c>
       <c r="C9" t="n">
-        <v>0.9501289523463659</v>
+        <v>0.9627152083157438</v>
       </c>
       <c r="D9" t="n">
         <v>0.9122368314914899</v>
@@ -585,10 +585,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1.10671601353631</v>
+        <v>1.09049422763081</v>
       </c>
       <c r="C10" t="n">
-        <v>1.052488714853364</v>
+        <v>1.038728786418037</v>
       </c>
       <c r="D10" t="n">
         <v>1.09620656114599</v>
@@ -617,10 +617,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-70.87753623188405</v>
+        <v>-71.931884057971</v>
       </c>
       <c r="C12" t="n">
-        <v>-31.20371640238972</v>
+        <v>-31.61706867511699</v>
       </c>
       <c r="D12" t="n">
         <v>-67.7185628742515</v>
@@ -633,10 +633,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3.754676258992806</v>
+        <v>3.231294964028778</v>
       </c>
       <c r="C13" t="n">
-        <v>1.079626828387301</v>
+        <v>0.8071549182749416</v>
       </c>
       <c r="D13" t="n">
         <v>3.306990881458967</v>
@@ -681,10 +681,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>58.08164990859233</v>
+        <v>49.9853861974406</v>
       </c>
       <c r="C16" t="n">
-        <v>32.08016381818381</v>
+        <v>23.98390010703208</v>
       </c>
       <c r="D16" t="n">
         <v>60.54113345521024</v>
@@ -780,7 +780,7 @@
         <v>0</v>
       </c>
       <c r="C22" t="n">
-        <v>-7.524090654205338</v>
+        <v>-153.0240906542052</v>
       </c>
       <c r="D22" t="n">
         <v>-97</v>
@@ -793,10 +793,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.7338817408422977</v>
+        <v>0.6315826478239472</v>
       </c>
       <c r="C23" t="n">
-        <v>0.499329395160896</v>
+        <v>0.3733106352547821</v>
       </c>
       <c r="D23" t="n">
         <v>0.9196956889264581</v>
@@ -11134,10 +11134,10 @@
         <v>46142</v>
       </c>
       <c r="B396" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C396" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D396" t="n">
         <v>575</v>
@@ -11146,10 +11146,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F396" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G396" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H396" t="n">
         <v>-610</v>
@@ -11160,10 +11160,10 @@
         <v>46143</v>
       </c>
       <c r="B397" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C397" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D397" t="n">
         <v>575</v>
@@ -11172,10 +11172,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F397" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G397" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H397" t="n">
         <v>-610</v>
@@ -11186,10 +11186,10 @@
         <v>46144</v>
       </c>
       <c r="B398" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C398" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D398" t="n">
         <v>575</v>
@@ -11198,10 +11198,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F398" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G398" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H398" t="n">
         <v>-610</v>
@@ -11212,10 +11212,10 @@
         <v>46145</v>
       </c>
       <c r="B399" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C399" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D399" t="n">
         <v>575</v>
@@ -11224,10 +11224,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F399" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G399" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H399" t="n">
         <v>-610</v>
@@ -11238,10 +11238,10 @@
         <v>46146</v>
       </c>
       <c r="B400" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C400" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D400" t="n">
         <v>457</v>
@@ -11250,10 +11250,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F400" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G400" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H400" t="n">
         <v>-728</v>
@@ -11264,10 +11264,10 @@
         <v>46147</v>
       </c>
       <c r="B401" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C401" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D401" t="n">
         <v>417</v>
@@ -11276,10 +11276,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F401" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G401" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H401" t="n">
         <v>-768</v>
@@ -11290,10 +11290,10 @@
         <v>46148</v>
       </c>
       <c r="B402" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C402" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D402" t="n">
         <v>326</v>
@@ -11302,10 +11302,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F402" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G402" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H402" t="n">
         <v>-859</v>
@@ -11316,10 +11316,10 @@
         <v>46149</v>
       </c>
       <c r="B403" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C403" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D403" t="n">
         <v>326</v>
@@ -11328,10 +11328,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F403" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G403" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H403" t="n">
         <v>-859</v>
@@ -11342,10 +11342,10 @@
         <v>46150</v>
       </c>
       <c r="B404" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C404" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D404" t="n">
         <v>255</v>
@@ -11354,10 +11354,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F404" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G404" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H404" t="n">
         <v>-930</v>
@@ -11368,10 +11368,10 @@
         <v>46151</v>
       </c>
       <c r="B405" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C405" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D405" t="n">
         <v>255</v>
@@ -11380,10 +11380,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F405" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G405" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H405" t="n">
         <v>-930</v>
@@ -11394,10 +11394,10 @@
         <v>46152</v>
       </c>
       <c r="B406" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C406" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D406" t="n">
         <v>255</v>
@@ -11406,10 +11406,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F406" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G406" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H406" t="n">
         <v>-930</v>
@@ -11420,10 +11420,10 @@
         <v>46153</v>
       </c>
       <c r="B407" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C407" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D407" t="n">
         <v>255</v>
@@ -11432,10 +11432,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F407" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G407" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H407" t="n">
         <v>-930</v>
@@ -11446,10 +11446,10 @@
         <v>46154</v>
       </c>
       <c r="B408" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C408" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D408" t="n">
         <v>495</v>
@@ -11458,10 +11458,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F408" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G408" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H408" t="n">
         <v>-690</v>
@@ -11472,10 +11472,10 @@
         <v>46155</v>
       </c>
       <c r="B409" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C409" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D409" t="n">
         <v>495</v>
@@ -11484,10 +11484,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F409" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G409" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H409" t="n">
         <v>-690</v>
@@ -11498,10 +11498,10 @@
         <v>46156</v>
       </c>
       <c r="B410" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C410" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D410" t="n">
         <v>360</v>
@@ -11510,10 +11510,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F410" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G410" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H410" t="n">
         <v>-825</v>
@@ -11524,10 +11524,10 @@
         <v>46157</v>
       </c>
       <c r="B411" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C411" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D411" t="n">
         <v>220</v>
@@ -11536,10 +11536,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F411" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G411" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H411" t="n">
         <v>-965</v>
@@ -11550,10 +11550,10 @@
         <v>46158</v>
       </c>
       <c r="B412" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C412" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D412" t="n">
         <v>220</v>
@@ -11562,10 +11562,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F412" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G412" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H412" t="n">
         <v>-965</v>
@@ -11576,10 +11576,10 @@
         <v>46159</v>
       </c>
       <c r="B413" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C413" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D413" t="n">
         <v>220</v>
@@ -11588,10 +11588,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F413" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G413" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H413" t="n">
         <v>-965</v>
@@ -11602,10 +11602,10 @@
         <v>46160</v>
       </c>
       <c r="B414" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C414" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D414" t="n">
         <v>220</v>
@@ -11614,10 +11614,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F414" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G414" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H414" t="n">
         <v>-965</v>
@@ -11628,10 +11628,10 @@
         <v>46161</v>
       </c>
       <c r="B415" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C415" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D415" t="n">
         <v>153</v>
@@ -11640,10 +11640,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F415" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G415" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H415" t="n">
         <v>-1032</v>
@@ -11654,10 +11654,10 @@
         <v>46162</v>
       </c>
       <c r="B416" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C416" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D416" t="n">
         <v>105</v>
@@ -11666,10 +11666,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F416" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G416" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H416" t="n">
         <v>-1080</v>
@@ -11680,10 +11680,10 @@
         <v>46163</v>
       </c>
       <c r="B417" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C417" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D417" t="n">
         <v>105</v>
@@ -11692,10 +11692,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F417" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G417" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H417" t="n">
         <v>-1080</v>
@@ -11706,10 +11706,10 @@
         <v>46164</v>
       </c>
       <c r="B418" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C418" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D418" t="n">
         <v>105</v>
@@ -11718,10 +11718,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F418" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G418" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H418" t="n">
         <v>-1080</v>
@@ -11732,10 +11732,10 @@
         <v>46165</v>
       </c>
       <c r="B419" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C419" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D419" t="n">
         <v>105</v>
@@ -11744,10 +11744,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F419" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G419" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H419" t="n">
         <v>-1080</v>
@@ -11758,10 +11758,10 @@
         <v>46166</v>
       </c>
       <c r="B420" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C420" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D420" t="n">
         <v>105</v>
@@ -11770,10 +11770,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F420" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G420" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H420" t="n">
         <v>-1080</v>
@@ -11784,10 +11784,10 @@
         <v>46167</v>
       </c>
       <c r="B421" t="n">
-        <v>-59.09999999999992</v>
+        <v>-204.5999999999999</v>
       </c>
       <c r="C421" t="n">
-        <v>-302.7262829869759</v>
+        <v>-448.2262829869759</v>
       </c>
       <c r="D421" t="n">
         <v>105</v>
@@ -11796,10 +11796,10 @@
         <v>-243.6262829869762</v>
       </c>
       <c r="F421" t="n">
-        <v>-860.8000000000001</v>
+        <v>-1006.3</v>
       </c>
       <c r="G421" t="n">
-        <v>-886.7710999999998</v>
+        <v>-1032.2711</v>
       </c>
       <c r="H421" t="n">
         <v>-1080</v>
@@ -11810,10 +11810,10 @@
         <v>46168</v>
       </c>
       <c r="B422" t="n">
-        <v>2.500000000000092</v>
+        <v>-142.9999999999999</v>
       </c>
       <c r="C422" t="n">
-        <v>-241.2562829869759</v>
+        <v>-386.7562829869759</v>
       </c>
       <c r="D422" t="n">
         <v>168</v>
@@ -11822,10 +11822,10 @@
         <v>-243.7562829869761</v>
       </c>
       <c r="F422" t="n">
-        <v>-799.2</v>
+        <v>-944.7</v>
       </c>
       <c r="G422" t="n">
-        <v>-825.3010999999998</v>
+        <v>-970.8010999999998</v>
       </c>
       <c r="H422" t="n">
         <v>-1017</v>
@@ -11836,10 +11836,10 @@
         <v>46169</v>
       </c>
       <c r="B423" t="n">
-        <v>2.500000000000092</v>
+        <v>-142.9999999999999</v>
       </c>
       <c r="C423" t="n">
-        <v>-242.5262829869759</v>
+        <v>-388.0262829869758</v>
       </c>
       <c r="D423" t="n">
         <v>168</v>
@@ -11848,10 +11848,10 @@
         <v>-245.0262829869762</v>
       </c>
       <c r="F423" t="n">
-        <v>-799.2</v>
+        <v>-944.7</v>
       </c>
       <c r="G423" t="n">
-        <v>-826.5710999999999</v>
+        <v>-972.0710999999998</v>
       </c>
       <c r="H423" t="n">
         <v>-1017</v>
@@ -11862,10 +11862,10 @@
         <v>46170</v>
       </c>
       <c r="B424" t="n">
-        <v>2.500000000000092</v>
+        <v>-142.9999999999999</v>
       </c>
       <c r="C424" t="n">
-        <v>-242.5262829869759</v>
+        <v>-388.0262829869758</v>
       </c>
       <c r="D424" t="n">
         <v>168</v>
@@ -11874,10 +11874,10 @@
         <v>-245.0262829869762</v>
       </c>
       <c r="F424" t="n">
-        <v>-799.2</v>
+        <v>-944.7</v>
       </c>
       <c r="G424" t="n">
-        <v>-826.5710999999999</v>
+        <v>-972.0710999999998</v>
       </c>
       <c r="H424" t="n">
         <v>-1017</v>
@@ -11888,10 +11888,10 @@
         <v>46171</v>
       </c>
       <c r="B425" t="n">
-        <v>31.70000000000009</v>
+        <v>-113.7999999999999</v>
       </c>
       <c r="C425" t="n">
-        <v>-213.5169371925834</v>
+        <v>-359.0169371925833</v>
       </c>
       <c r="D425" t="n">
         <v>199</v>
@@ -11900,10 +11900,10 @@
         <v>-245.2169371925836</v>
       </c>
       <c r="F425" t="n">
-        <v>-770.0000000000001</v>
+        <v>-915.5</v>
       </c>
       <c r="G425" t="n">
-        <v>-797.5617542056073</v>
+        <v>-943.0617542056073</v>
       </c>
       <c r="H425" t="n">
         <v>-986</v>
@@ -11914,10 +11914,10 @@
         <v>46172</v>
       </c>
       <c r="B426" t="n">
-        <v>31.70000000000009</v>
+        <v>-113.7999999999999</v>
       </c>
       <c r="C426" t="n">
-        <v>-213.5169371925834</v>
+        <v>-359.0169371925833</v>
       </c>
       <c r="D426" t="n">
         <v>199</v>
@@ -11926,10 +11926,10 @@
         <v>-245.2169371925836</v>
       </c>
       <c r="F426" t="n">
-        <v>-770.0000000000001</v>
+        <v>-915.5</v>
       </c>
       <c r="G426" t="n">
-        <v>-797.5617542056073</v>
+        <v>-943.0617542056073</v>
       </c>
       <c r="H426" t="n">
         <v>-986</v>
@@ -11940,10 +11940,10 @@
         <v>46173</v>
       </c>
       <c r="B427" t="n">
-        <v>31.70000000000009</v>
+        <v>-113.7999999999999</v>
       </c>
       <c r="C427" t="n">
-        <v>-213.5169371925834</v>
+        <v>-359.0169371925833</v>
       </c>
       <c r="D427" t="n">
         <v>199</v>
@@ -11952,10 +11952,10 @@
         <v>-245.2169371925836</v>
       </c>
       <c r="F427" t="n">
-        <v>-770.0000000000001</v>
+        <v>-915.5</v>
       </c>
       <c r="G427" t="n">
-        <v>-797.5617542056073</v>
+        <v>-943.0617542056073</v>
       </c>
       <c r="H427" t="n">
         <v>-986</v>
@@ -11966,10 +11966,10 @@
         <v>46174</v>
       </c>
       <c r="B428" t="n">
-        <v>152.0000000000001</v>
+        <v>6.500000000000114</v>
       </c>
       <c r="C428" t="n">
-        <v>-93.21693719258339</v>
+        <v>-238.7169371925833</v>
       </c>
       <c r="D428" t="n">
         <v>318</v>
@@ -11978,10 +11978,10 @@
         <v>-245.2169371925836</v>
       </c>
       <c r="F428" t="n">
-        <v>-649.7</v>
+        <v>-795.2</v>
       </c>
       <c r="G428" t="n">
-        <v>-677.2617542056073</v>
+        <v>-822.7617542056073</v>
       </c>
       <c r="H428" t="n">
         <v>-867</v>
@@ -11992,10 +11992,10 @@
         <v>46175</v>
       </c>
       <c r="B429" t="n">
-        <v>55.80000000000008</v>
+        <v>-89.69999999999989</v>
       </c>
       <c r="C429" t="n">
-        <v>-191.8440399963217</v>
+        <v>-337.3440399963216</v>
       </c>
       <c r="D429" t="n">
         <v>221</v>
@@ -12004,10 +12004,10 @@
         <v>-247.6440399963219</v>
       </c>
       <c r="F429" t="n">
-        <v>-745.9000000000001</v>
+        <v>-891.4000000000001</v>
       </c>
       <c r="G429" t="n">
-        <v>-775.8888570093457</v>
+        <v>-921.3888570093455</v>
       </c>
       <c r="H429" t="n">
         <v>-964</v>
@@ -12018,10 +12018,10 @@
         <v>46176</v>
       </c>
       <c r="B430" t="n">
-        <v>55.80000000000008</v>
+        <v>-89.69999999999989</v>
       </c>
       <c r="C430" t="n">
-        <v>-197.5840399963217</v>
+        <v>-343.0840399963216</v>
       </c>
       <c r="D430" t="n">
         <v>221</v>
@@ -12030,10 +12030,10 @@
         <v>-253.3840399963219</v>
       </c>
       <c r="F430" t="n">
-        <v>-745.9000000000001</v>
+        <v>-891.4000000000001</v>
       </c>
       <c r="G430" t="n">
-        <v>-781.6288570093457</v>
+        <v>-927.1288570093456</v>
       </c>
       <c r="H430" t="n">
         <v>-964</v>
@@ -12044,10 +12044,10 @@
         <v>46177</v>
       </c>
       <c r="B431" t="n">
-        <v>55.80000000000008</v>
+        <v>-89.69999999999989</v>
       </c>
       <c r="C431" t="n">
-        <v>-204.7140399963217</v>
+        <v>-350.2140399963216</v>
       </c>
       <c r="D431" t="n">
         <v>221</v>
@@ -12056,10 +12056,10 @@
         <v>-260.514039996322</v>
       </c>
       <c r="F431" t="n">
-        <v>-745.9000000000001</v>
+        <v>-891.4000000000001</v>
       </c>
       <c r="G431" t="n">
-        <v>-788.7588570093457</v>
+        <v>-934.2588570093455</v>
       </c>
       <c r="H431" t="n">
         <v>-964</v>
@@ -12070,10 +12070,10 @@
         <v>46178</v>
       </c>
       <c r="B432" t="n">
-        <v>126.2000000000001</v>
+        <v>-19.29999999999988</v>
       </c>
       <c r="C432" t="n">
-        <v>-131.6140399963217</v>
+        <v>-277.1140399963216</v>
       </c>
       <c r="D432" t="n">
         <v>292</v>
@@ -12082,10 +12082,10 @@
         <v>-257.814039996322</v>
       </c>
       <c r="F432" t="n">
-        <v>-675.5000000000001</v>
+        <v>-821</v>
       </c>
       <c r="G432" t="n">
-        <v>-715.6588570093456</v>
+        <v>-861.1588570093455</v>
       </c>
       <c r="H432" t="n">
         <v>-893</v>
@@ -12096,10 +12096,10 @@
         <v>46179</v>
       </c>
       <c r="B433" t="n">
-        <v>126.2000000000001</v>
+        <v>-19.29999999999988</v>
       </c>
       <c r="C433" t="n">
-        <v>-131.6140399963217</v>
+        <v>-277.1140399963216</v>
       </c>
       <c r="D433" t="n">
         <v>292</v>
@@ -12108,10 +12108,10 @@
         <v>-257.814039996322</v>
       </c>
       <c r="F433" t="n">
-        <v>-675.5000000000001</v>
+        <v>-821</v>
       </c>
       <c r="G433" t="n">
-        <v>-715.6588570093456</v>
+        <v>-861.1588570093455</v>
       </c>
       <c r="H433" t="n">
         <v>-893</v>
@@ -12122,10 +12122,10 @@
         <v>46180</v>
       </c>
       <c r="B434" t="n">
-        <v>126.2000000000001</v>
+        <v>-19.29999999999988</v>
       </c>
       <c r="C434" t="n">
-        <v>-131.6140399963217</v>
+        <v>-277.1140399963216</v>
       </c>
       <c r="D434" t="n">
         <v>292</v>
@@ -12134,10 +12134,10 @@
         <v>-257.814039996322</v>
       </c>
       <c r="F434" t="n">
-        <v>-675.5000000000001</v>
+        <v>-821</v>
       </c>
       <c r="G434" t="n">
-        <v>-715.6588570093456</v>
+        <v>-861.1588570093455</v>
       </c>
       <c r="H434" t="n">
         <v>-893</v>
@@ -12148,10 +12148,10 @@
         <v>46181</v>
       </c>
       <c r="B435" t="n">
-        <v>126.2000000000001</v>
+        <v>-19.29999999999988</v>
       </c>
       <c r="C435" t="n">
-        <v>-140.5140399963217</v>
+        <v>-286.0140399963216</v>
       </c>
       <c r="D435" t="n">
         <v>292</v>
@@ -12160,10 +12160,10 @@
         <v>-266.714039996322</v>
       </c>
       <c r="F435" t="n">
-        <v>-675.5000000000001</v>
+        <v>-821</v>
       </c>
       <c r="G435" t="n">
-        <v>-724.5588570093456</v>
+        <v>-870.0588570093455</v>
       </c>
       <c r="H435" t="n">
         <v>-893</v>
@@ -12174,10 +12174,10 @@
         <v>46182</v>
       </c>
       <c r="B436" t="n">
-        <v>296.4000000000001</v>
+        <v>150.9000000000001</v>
       </c>
       <c r="C436" t="n">
-        <v>26.88596000367826</v>
+        <v>-118.6140399963216</v>
       </c>
       <c r="D436" t="n">
         <v>466</v>
@@ -12186,10 +12186,10 @@
         <v>-269.514039996322</v>
       </c>
       <c r="F436" t="n">
-        <v>-505.3000000000001</v>
+        <v>-650.8000000000001</v>
       </c>
       <c r="G436" t="n">
-        <v>-557.1588570093456</v>
+        <v>-702.6588570093455</v>
       </c>
       <c r="H436" t="n">
         <v>-719</v>
@@ -12200,10 +12200,10 @@
         <v>46183</v>
       </c>
       <c r="B437" t="n">
-        <v>169.3000000000001</v>
+        <v>23.8000000000001</v>
       </c>
       <c r="C437" t="n">
-        <v>-97.52403999632173</v>
+        <v>-243.0240399963216</v>
       </c>
       <c r="D437" t="n">
         <v>330</v>
@@ -12212,10 +12212,10 @@
         <v>-266.824039996322</v>
       </c>
       <c r="F437" t="n">
-        <v>-632.4000000000001</v>
+        <v>-777.9000000000001</v>
       </c>
       <c r="G437" t="n">
-        <v>-681.5688570093457</v>
+        <v>-827.0688570093455</v>
       </c>
       <c r="H437" t="n">
         <v>-855</v>
@@ -12226,10 +12226,10 @@
         <v>46184</v>
       </c>
       <c r="B438" t="n">
-        <v>121.9000000000001</v>
+        <v>-23.5999999999999</v>
       </c>
       <c r="C438" t="n">
-        <v>-147.5740399963217</v>
+        <v>-293.0740399963216</v>
       </c>
       <c r="D438" t="n">
         <v>280</v>
@@ -12238,10 +12238,10 @@
         <v>-269.4740399963219</v>
       </c>
       <c r="F438" t="n">
-        <v>-679.8000000000001</v>
+        <v>-825.3000000000001</v>
       </c>
       <c r="G438" t="n">
-        <v>-731.6188570093457</v>
+        <v>-877.1188570093454</v>
       </c>
       <c r="H438" t="n">
         <v>-905</v>
@@ -12252,10 +12252,10 @@
         <v>46185</v>
       </c>
       <c r="B439" t="n">
-        <v>121.9000000000001</v>
+        <v>-23.5999999999999</v>
       </c>
       <c r="C439" t="n">
-        <v>-147.5740399963217</v>
+        <v>-293.0740399963216</v>
       </c>
       <c r="D439" t="n">
         <v>280</v>
@@ -12264,10 +12264,10 @@
         <v>-269.4740399963219</v>
       </c>
       <c r="F439" t="n">
-        <v>-679.8000000000001</v>
+        <v>-825.3000000000001</v>
       </c>
       <c r="G439" t="n">
-        <v>-731.6188570093457</v>
+        <v>-877.1188570093454</v>
       </c>
       <c r="H439" t="n">
         <v>-905</v>
@@ -12278,10 +12278,10 @@
         <v>46186</v>
       </c>
       <c r="B440" t="n">
-        <v>121.9000000000001</v>
+        <v>-23.5999999999999</v>
       </c>
       <c r="C440" t="n">
-        <v>-147.5740399963217</v>
+        <v>-293.0740399963216</v>
       </c>
       <c r="D440" t="n">
         <v>280</v>
@@ -12290,10 +12290,10 @@
         <v>-269.4740399963219</v>
       </c>
       <c r="F440" t="n">
-        <v>-679.8000000000001</v>
+        <v>-825.3000000000001</v>
       </c>
       <c r="G440" t="n">
-        <v>-731.6188570093457</v>
+        <v>-877.1188570093454</v>
       </c>
       <c r="H440" t="n">
         <v>-905</v>
@@ -12304,10 +12304,10 @@
         <v>46187</v>
       </c>
       <c r="B441" t="n">
-        <v>121.9000000000001</v>
+        <v>-23.5999999999999</v>
       </c>
       <c r="C441" t="n">
-        <v>-147.5740399963217</v>
+        <v>-293.0740399963216</v>
       </c>
       <c r="D441" t="n">
         <v>280</v>
@@ -12316,10 +12316,10 @@
         <v>-269.4740399963219</v>
       </c>
       <c r="F441" t="n">
-        <v>-679.8000000000001</v>
+        <v>-825.3000000000001</v>
       </c>
       <c r="G441" t="n">
-        <v>-731.6188570093457</v>
+        <v>-877.1188570093454</v>
       </c>
       <c r="H441" t="n">
         <v>-905</v>
@@ -12330,10 +12330,10 @@
         <v>46188</v>
       </c>
       <c r="B442" t="n">
-        <v>121.9000000000001</v>
+        <v>-23.5999999999999</v>
       </c>
       <c r="C442" t="n">
-        <v>-156.5340399963218</v>
+        <v>-302.0340399963216</v>
       </c>
       <c r="D442" t="n">
         <v>280</v>
@@ -12342,10 +12342,10 @@
         <v>-278.4340399963219</v>
       </c>
       <c r="F442" t="n">
-        <v>-679.8000000000001</v>
+        <v>-825.3000000000001</v>
       </c>
       <c r="G442" t="n">
-        <v>-740.5788570093457</v>
+        <v>-886.0788570093455</v>
       </c>
       <c r="H442" t="n">
         <v>-905</v>
@@ -12356,10 +12356,10 @@
         <v>46189</v>
       </c>
       <c r="B443" t="n">
-        <v>298.5000000000001</v>
+        <v>153.0000000000001</v>
       </c>
       <c r="C443" t="n">
-        <v>14.84596000367827</v>
+        <v>-130.6540399963215</v>
       </c>
       <c r="D443" t="n">
         <v>469</v>
@@ -12368,10 +12368,10 @@
         <v>-283.654039996322</v>
       </c>
       <c r="F443" t="n">
-        <v>-503.2</v>
+        <v>-648.7</v>
       </c>
       <c r="G443" t="n">
-        <v>-569.1988570093456</v>
+        <v>-714.6988570093455</v>
       </c>
       <c r="H443" t="n">
         <v>-716</v>
@@ -12382,10 +12382,10 @@
         <v>46190</v>
       </c>
       <c r="B444" t="n">
-        <v>298.5000000000001</v>
+        <v>153.0000000000001</v>
       </c>
       <c r="C444" t="n">
-        <v>11.79596000367827</v>
+        <v>-133.7040399963215</v>
       </c>
       <c r="D444" t="n">
         <v>469</v>
@@ -12394,10 +12394,10 @@
         <v>-286.704039996322</v>
       </c>
       <c r="F444" t="n">
-        <v>-503.2</v>
+        <v>-648.7</v>
       </c>
       <c r="G444" t="n">
-        <v>-572.2488570093457</v>
+        <v>-717.7488570093454</v>
       </c>
       <c r="H444" t="n">
         <v>-716</v>
@@ -12408,10 +12408,10 @@
         <v>46191</v>
       </c>
       <c r="B445" t="n">
-        <v>298.5000000000001</v>
+        <v>153.0000000000001</v>
       </c>
       <c r="C445" t="n">
-        <v>6.855960003678271</v>
+        <v>-138.6440399963215</v>
       </c>
       <c r="D445" t="n">
         <v>469</v>
@@ -12420,10 +12420,10 @@
         <v>-291.644039996322</v>
       </c>
       <c r="F445" t="n">
-        <v>-503.2</v>
+        <v>-648.7</v>
       </c>
       <c r="G445" t="n">
-        <v>-577.1888570093456</v>
+        <v>-722.6888570093455</v>
       </c>
       <c r="H445" t="n">
         <v>-716</v>
@@ -12434,10 +12434,10 @@
         <v>46192</v>
       </c>
       <c r="B446" t="n">
-        <v>298.5000000000001</v>
+        <v>153.0000000000001</v>
       </c>
       <c r="C446" t="n">
-        <v>10.19596000367827</v>
+        <v>-135.3040399963215</v>
       </c>
       <c r="D446" t="n">
         <v>469</v>
@@ -12446,10 +12446,10 @@
         <v>-288.304039996322</v>
       </c>
       <c r="F446" t="n">
-        <v>-503.2</v>
+        <v>-648.7</v>
       </c>
       <c r="G446" t="n">
-        <v>-573.8488570093457</v>
+        <v>-719.3488570093455</v>
       </c>
       <c r="H446" t="n">
         <v>-716</v>
@@ -12460,10 +12460,10 @@
         <v>46193</v>
       </c>
       <c r="B447" t="n">
-        <v>298.5000000000001</v>
+        <v>153.0000000000001</v>
       </c>
       <c r="C447" t="n">
-        <v>10.19596000367827</v>
+        <v>-135.3040399963215</v>
       </c>
       <c r="D447" t="n">
         <v>469</v>
@@ -12472,10 +12472,10 @@
         <v>-288.304039996322</v>
       </c>
       <c r="F447" t="n">
-        <v>-503.2</v>
+        <v>-648.7</v>
       </c>
       <c r="G447" t="n">
-        <v>-573.8488570093457</v>
+        <v>-719.3488570093455</v>
       </c>
       <c r="H447" t="n">
         <v>-716</v>
@@ -12486,10 +12486,10 @@
         <v>46194</v>
       </c>
       <c r="B448" t="n">
-        <v>298.5000000000001</v>
+        <v>153.0000000000001</v>
       </c>
       <c r="C448" t="n">
-        <v>10.19596000367827</v>
+        <v>-135.3040399963215</v>
       </c>
       <c r="D448" t="n">
         <v>469</v>
@@ -12498,10 +12498,10 @@
         <v>-288.304039996322</v>
       </c>
       <c r="F448" t="n">
-        <v>-503.2</v>
+        <v>-648.7</v>
       </c>
       <c r="G448" t="n">
-        <v>-573.8488570093457</v>
+        <v>-719.3488570093455</v>
       </c>
       <c r="H448" t="n">
         <v>-716</v>
@@ -12512,10 +12512,10 @@
         <v>46195</v>
       </c>
       <c r="B449" t="n">
-        <v>298.5000000000001</v>
+        <v>153.0000000000001</v>
       </c>
       <c r="C449" t="n">
-        <v>6.395960003678272</v>
+        <v>-139.1040399963215</v>
       </c>
       <c r="D449" t="n">
         <v>469</v>
@@ -12524,10 +12524,10 @@
         <v>-292.104039996322</v>
       </c>
       <c r="F449" t="n">
-        <v>-503.2</v>
+        <v>-648.7</v>
       </c>
       <c r="G449" t="n">
-        <v>-577.6488570093456</v>
+        <v>-723.1488570093454</v>
       </c>
       <c r="H449" t="n">
         <v>-716</v>
@@ -12538,10 +12538,10 @@
         <v>46196</v>
       </c>
       <c r="B450" t="n">
-        <v>407.7000000000001</v>
+        <v>262.2000000000001</v>
       </c>
       <c r="C450" t="n">
-        <v>112.9859600036783</v>
+        <v>-32.51403999632154</v>
       </c>
       <c r="D450" t="n">
         <v>584</v>
@@ -12550,10 +12550,10 @@
         <v>-294.714039996322</v>
       </c>
       <c r="F450" t="n">
-        <v>-394.0000000000001</v>
+        <v>-539.5</v>
       </c>
       <c r="G450" t="n">
-        <v>-471.0588570093457</v>
+        <v>-616.5588570093455</v>
       </c>
       <c r="H450" t="n">
         <v>-601</v>
@@ -12564,10 +12564,10 @@
         <v>46197</v>
       </c>
       <c r="B451" t="n">
-        <v>392.7000000000001</v>
+        <v>247.2000000000001</v>
       </c>
       <c r="C451" t="n">
-        <v>95.42596000367827</v>
+        <v>-50.07403999632155</v>
       </c>
       <c r="D451" t="n">
         <v>557</v>
@@ -12576,10 +12576,10 @@
         <v>-297.274039996322</v>
       </c>
       <c r="F451" t="n">
-        <v>-409.0000000000001</v>
+        <v>-554.5</v>
       </c>
       <c r="G451" t="n">
-        <v>-488.6188570093457</v>
+        <v>-634.1188570093454</v>
       </c>
       <c r="H451" t="n">
         <v>-628</v>
@@ -12590,10 +12590,10 @@
         <v>46198</v>
       </c>
       <c r="B452" t="n">
-        <v>392.7000000000001</v>
+        <v>247.2000000000001</v>
       </c>
       <c r="C452" t="n">
-        <v>91.82596000367828</v>
+        <v>-53.67403999632155</v>
       </c>
       <c r="D452" t="n">
         <v>557</v>
@@ -12602,10 +12602,10 @@
         <v>-300.874039996322</v>
       </c>
       <c r="F452" t="n">
-        <v>-409.0000000000001</v>
+        <v>-554.5</v>
       </c>
       <c r="G452" t="n">
-        <v>-492.2188570093456</v>
+        <v>-637.7188570093455</v>
       </c>
       <c r="H452" t="n">
         <v>-628</v>
@@ -12616,10 +12616,10 @@
         <v>46199</v>
       </c>
       <c r="B453" t="n">
-        <v>392.7000000000001</v>
+        <v>247.2000000000001</v>
       </c>
       <c r="C453" t="n">
-        <v>91.82596000367828</v>
+        <v>-53.67403999632155</v>
       </c>
       <c r="D453" t="n">
         <v>557</v>
@@ -12628,10 +12628,10 @@
         <v>-300.874039996322</v>
       </c>
       <c r="F453" t="n">
-        <v>-409.0000000000001</v>
+        <v>-554.5</v>
       </c>
       <c r="G453" t="n">
-        <v>-492.2188570093456</v>
+        <v>-637.7188570093455</v>
       </c>
       <c r="H453" t="n">
         <v>-628</v>
@@ -12642,10 +12642,10 @@
         <v>46200</v>
       </c>
       <c r="B454" t="n">
-        <v>392.7000000000001</v>
+        <v>247.2000000000001</v>
       </c>
       <c r="C454" t="n">
-        <v>91.82596000367828</v>
+        <v>-53.67403999632155</v>
       </c>
       <c r="D454" t="n">
         <v>557</v>
@@ -12654,10 +12654,10 @@
         <v>-300.874039996322</v>
       </c>
       <c r="F454" t="n">
-        <v>-409.0000000000001</v>
+        <v>-554.5</v>
       </c>
       <c r="G454" t="n">
-        <v>-492.2188570093456</v>
+        <v>-637.7188570093455</v>
       </c>
       <c r="H454" t="n">
         <v>-628</v>
@@ -12668,10 +12668,10 @@
         <v>46201</v>
       </c>
       <c r="B455" t="n">
-        <v>392.7000000000001</v>
+        <v>247.2000000000001</v>
       </c>
       <c r="C455" t="n">
-        <v>91.82596000367828</v>
+        <v>-53.67403999632155</v>
       </c>
       <c r="D455" t="n">
         <v>557</v>
@@ -12680,10 +12680,10 @@
         <v>-300.874039996322</v>
       </c>
       <c r="F455" t="n">
-        <v>-409.0000000000001</v>
+        <v>-554.5</v>
       </c>
       <c r="G455" t="n">
-        <v>-492.2188570093456</v>
+        <v>-637.7188570093455</v>
       </c>
       <c r="H455" t="n">
         <v>-628</v>
@@ -12694,10 +12694,10 @@
         <v>46202</v>
       </c>
       <c r="B456" t="n">
-        <v>478.4000000000001</v>
+        <v>332.9000000000001</v>
       </c>
       <c r="C456" t="n">
-        <v>175.0259600036783</v>
+        <v>29.52596000367846</v>
       </c>
       <c r="D456" t="n">
         <v>572</v>
@@ -12706,10 +12706,10 @@
         <v>-303.374039996322</v>
       </c>
       <c r="F456" t="n">
-        <v>-323.3000000000001</v>
+        <v>-468.8000000000001</v>
       </c>
       <c r="G456" t="n">
-        <v>-409.0188570093457</v>
+        <v>-554.5188570093454</v>
       </c>
       <c r="H456" t="n">
         <v>-613</v>
@@ -12720,10 +12720,10 @@
         <v>46203</v>
       </c>
       <c r="B457" t="n">
-        <v>507.4000000000001</v>
+        <v>361.9000000000001</v>
       </c>
       <c r="C457" t="n">
-        <v>201.7359600036783</v>
+        <v>56.23596000367846</v>
       </c>
       <c r="D457" t="n">
         <v>650</v>
@@ -12732,10 +12732,10 @@
         <v>-305.6640399963221</v>
       </c>
       <c r="F457" t="n">
-        <v>-294.3000000000001</v>
+        <v>-439.8000000000001</v>
       </c>
       <c r="G457" t="n">
-        <v>-382.3088570093456</v>
+        <v>-527.8088570093455</v>
       </c>
       <c r="H457" t="n">
         <v>-535</v>
@@ -12746,10 +12746,10 @@
         <v>46204</v>
       </c>
       <c r="B458" t="n">
-        <v>465.1000000000001</v>
+        <v>319.6000000000001</v>
       </c>
       <c r="C458" t="n">
-        <v>159.8859600036783</v>
+        <v>14.38596000367846</v>
       </c>
       <c r="D458" t="n">
         <v>608</v>
@@ -12758,10 +12758,10 @@
         <v>-305.2140399963221</v>
       </c>
       <c r="F458" t="n">
-        <v>-336.6000000000001</v>
+        <v>-482.1000000000001</v>
       </c>
       <c r="G458" t="n">
-        <v>-424.1588570093456</v>
+        <v>-569.6588570093454</v>
       </c>
       <c r="H458" t="n">
         <v>-577</v>
@@ -12772,10 +12772,10 @@
         <v>46205</v>
       </c>
       <c r="B459" t="n">
-        <v>465.1000000000001</v>
+        <v>319.6000000000001</v>
       </c>
       <c r="C459" t="n">
-        <v>158.8859600036783</v>
+        <v>13.38596000367846</v>
       </c>
       <c r="D459" t="n">
         <v>608</v>
@@ -12784,10 +12784,10 @@
         <v>-306.2140399963221</v>
       </c>
       <c r="F459" t="n">
-        <v>-336.6000000000001</v>
+        <v>-482.1000000000001</v>
       </c>
       <c r="G459" t="n">
-        <v>-425.1588570093456</v>
+        <v>-570.6588570093454</v>
       </c>
       <c r="H459" t="n">
         <v>-577</v>
@@ -12798,10 +12798,10 @@
         <v>46206</v>
       </c>
       <c r="B460" t="n">
-        <v>565.7</v>
+        <v>420.2</v>
       </c>
       <c r="C460" t="n">
-        <v>257.6859600036783</v>
+        <v>112.1859600036785</v>
       </c>
       <c r="D460" t="n">
         <v>608</v>
@@ -12810,10 +12810,10 @@
         <v>-308.0140399963221</v>
       </c>
       <c r="F460" t="n">
-        <v>-236.0000000000001</v>
+        <v>-381.5000000000001</v>
       </c>
       <c r="G460" t="n">
-        <v>-326.3588570093456</v>
+        <v>-471.8588570093455</v>
       </c>
       <c r="H460" t="n">
         <v>-577</v>
@@ -12824,10 +12824,10 @@
         <v>46207</v>
       </c>
       <c r="B461" t="n">
-        <v>565.7</v>
+        <v>420.2</v>
       </c>
       <c r="C461" t="n">
-        <v>257.6859600036783</v>
+        <v>112.1859600036785</v>
       </c>
       <c r="D461" t="n">
         <v>608</v>
@@ -12836,10 +12836,10 @@
         <v>-308.0140399963221</v>
       </c>
       <c r="F461" t="n">
-        <v>-236.0000000000001</v>
+        <v>-381.5000000000001</v>
       </c>
       <c r="G461" t="n">
-        <v>-326.3588570093456</v>
+        <v>-471.8588570093455</v>
       </c>
       <c r="H461" t="n">
         <v>-577</v>
@@ -12850,10 +12850,10 @@
         <v>46208</v>
       </c>
       <c r="B462" t="n">
-        <v>565.7</v>
+        <v>420.2</v>
       </c>
       <c r="C462" t="n">
-        <v>257.6859600036783</v>
+        <v>112.1859600036785</v>
       </c>
       <c r="D462" t="n">
         <v>608</v>
@@ -12862,10 +12862,10 @@
         <v>-308.0140399963221</v>
       </c>
       <c r="F462" t="n">
-        <v>-236.0000000000001</v>
+        <v>-381.5000000000001</v>
       </c>
       <c r="G462" t="n">
-        <v>-326.3588570093456</v>
+        <v>-471.8588570093455</v>
       </c>
       <c r="H462" t="n">
         <v>-577</v>
@@ -12876,10 +12876,10 @@
         <v>46209</v>
       </c>
       <c r="B463" t="n">
-        <v>565.7</v>
+        <v>420.2</v>
       </c>
       <c r="C463" t="n">
-        <v>255.8659600036783</v>
+        <v>110.3659600036785</v>
       </c>
       <c r="D463" t="n">
         <v>608</v>
@@ -12888,10 +12888,10 @@
         <v>-309.8340399963221</v>
       </c>
       <c r="F463" t="n">
-        <v>-236.0000000000001</v>
+        <v>-381.5000000000001</v>
       </c>
       <c r="G463" t="n">
-        <v>-328.1788570093456</v>
+        <v>-473.6788570093454</v>
       </c>
       <c r="H463" t="n">
         <v>-577</v>
@@ -12902,10 +12902,10 @@
         <v>46210</v>
       </c>
       <c r="B464" t="n">
-        <v>612.1</v>
+        <v>466.6</v>
       </c>
       <c r="C464" t="n">
-        <v>300.2359600036783</v>
+        <v>154.7359600036785</v>
       </c>
       <c r="D464" t="n">
         <v>707</v>
@@ -12914,10 +12914,10 @@
         <v>-311.864039996322</v>
       </c>
       <c r="F464" t="n">
-        <v>-189.6000000000001</v>
+        <v>-335.1000000000001</v>
       </c>
       <c r="G464" t="n">
-        <v>-283.8088570093456</v>
+        <v>-429.3088570093455</v>
       </c>
       <c r="H464" t="n">
         <v>-478</v>
@@ -12928,10 +12928,10 @@
         <v>46211</v>
       </c>
       <c r="B465" t="n">
-        <v>529.6</v>
+        <v>384.1</v>
       </c>
       <c r="C465" t="n">
-        <v>223.6359600036783</v>
+        <v>78.13596000367846</v>
       </c>
       <c r="D465" t="n">
         <v>628</v>
@@ -12940,10 +12940,10 @@
         <v>-305.9640399963221</v>
       </c>
       <c r="F465" t="n">
-        <v>-272.1000000000001</v>
+        <v>-417.6000000000001</v>
       </c>
       <c r="G465" t="n">
-        <v>-360.4088570093456</v>
+        <v>-505.9088570093455</v>
       </c>
       <c r="H465" t="n">
         <v>-557</v>
@@ -12954,10 +12954,10 @@
         <v>46212</v>
       </c>
       <c r="B466" t="n">
-        <v>565.5</v>
+        <v>420</v>
       </c>
       <c r="C466" t="n">
-        <v>255.3359600036783</v>
+        <v>109.8359600036785</v>
       </c>
       <c r="D466" t="n">
         <v>628</v>
@@ -12966,10 +12966,10 @@
         <v>-310.1640399963221</v>
       </c>
       <c r="F466" t="n">
-        <v>-236.2000000000002</v>
+        <v>-381.7000000000002</v>
       </c>
       <c r="G466" t="n">
-        <v>-328.7088570093456</v>
+        <v>-474.2088570093455</v>
       </c>
       <c r="H466" t="n">
         <v>-557</v>
@@ -12980,10 +12980,10 @@
         <v>46213</v>
       </c>
       <c r="B467" t="n">
-        <v>565.5</v>
+        <v>420</v>
       </c>
       <c r="C467" t="n">
-        <v>253.2859600036783</v>
+        <v>107.7859600036785</v>
       </c>
       <c r="D467" t="n">
         <v>663</v>
@@ -12992,10 +12992,10 @@
         <v>-312.2140399963221</v>
       </c>
       <c r="F467" t="n">
-        <v>-236.2000000000002</v>
+        <v>-381.7000000000002</v>
       </c>
       <c r="G467" t="n">
-        <v>-330.7588570093457</v>
+        <v>-476.2588570093454</v>
       </c>
       <c r="H467" t="n">
         <v>-522</v>
@@ -13006,10 +13006,10 @@
         <v>46214</v>
       </c>
       <c r="B468" t="n">
-        <v>565.5</v>
+        <v>420</v>
       </c>
       <c r="C468" t="n">
-        <v>253.2859600036783</v>
+        <v>107.7859600036785</v>
       </c>
       <c r="D468" t="n">
         <v>663</v>
@@ -13018,10 +13018,10 @@
         <v>-312.2140399963221</v>
       </c>
       <c r="F468" t="n">
-        <v>-236.2000000000002</v>
+        <v>-381.7000000000002</v>
       </c>
       <c r="G468" t="n">
-        <v>-330.7588570093457</v>
+        <v>-476.2588570093454</v>
       </c>
       <c r="H468" t="n">
         <v>-522</v>
@@ -13032,10 +13032,10 @@
         <v>46215</v>
       </c>
       <c r="B469" t="n">
-        <v>565.5</v>
+        <v>420</v>
       </c>
       <c r="C469" t="n">
-        <v>253.2859600036783</v>
+        <v>107.7859600036785</v>
       </c>
       <c r="D469" t="n">
         <v>663</v>
@@ -13044,10 +13044,10 @@
         <v>-312.2140399963221</v>
       </c>
       <c r="F469" t="n">
-        <v>-236.2000000000002</v>
+        <v>-381.7000000000002</v>
       </c>
       <c r="G469" t="n">
-        <v>-330.7588570093457</v>
+        <v>-476.2588570093454</v>
       </c>
       <c r="H469" t="n">
         <v>-522</v>
@@ -13058,10 +13058,10 @@
         <v>46216</v>
       </c>
       <c r="B470" t="n">
-        <v>434.6</v>
+        <v>289.1</v>
       </c>
       <c r="C470" t="n">
-        <v>117.9759600036783</v>
+        <v>-27.52403999632153</v>
       </c>
       <c r="D470" t="n">
         <v>529</v>
@@ -13070,10 +13070,10 @@
         <v>-316.6240399963221</v>
       </c>
       <c r="F470" t="n">
-        <v>-367.1000000000001</v>
+        <v>-512.6000000000001</v>
       </c>
       <c r="G470" t="n">
-        <v>-466.0688570093456</v>
+        <v>-611.5688570093455</v>
       </c>
       <c r="H470" t="n">
         <v>-656</v>
@@ -13084,10 +13084,10 @@
         <v>46217</v>
       </c>
       <c r="B471" t="n">
-        <v>411.6</v>
+        <v>266.1</v>
       </c>
       <c r="C471" t="n">
-        <v>98.9259600036783</v>
+        <v>-46.57403999632153</v>
       </c>
       <c r="D471" t="n">
         <v>513</v>
@@ -13096,10 +13096,10 @@
         <v>-312.6740399963221</v>
       </c>
       <c r="F471" t="n">
-        <v>-390.1000000000001</v>
+        <v>-535.6000000000001</v>
       </c>
       <c r="G471" t="n">
-        <v>-485.1188570093456</v>
+        <v>-630.6188570093454</v>
       </c>
       <c r="H471" t="n">
         <v>-672</v>
@@ -13110,10 +13110,10 @@
         <v>46218</v>
       </c>
       <c r="B472" t="n">
-        <v>263.7</v>
+        <v>118.2</v>
       </c>
       <c r="C472" t="n">
-        <v>-47.83403999632172</v>
+        <v>-193.3340399963216</v>
       </c>
       <c r="D472" t="n">
         <v>361</v>
@@ -13122,10 +13122,10 @@
         <v>-311.5340399963221</v>
       </c>
       <c r="F472" t="n">
-        <v>-538.0000000000001</v>
+        <v>-683.5000000000001</v>
       </c>
       <c r="G472" t="n">
-        <v>-631.8788570093457</v>
+        <v>-777.3788570093454</v>
       </c>
       <c r="H472" t="n">
         <v>-824</v>
@@ -13136,10 +13136,10 @@
         <v>46219</v>
       </c>
       <c r="B473" t="n">
-        <v>263.7</v>
+        <v>118.2</v>
       </c>
       <c r="C473" t="n">
-        <v>-51.70403999632172</v>
+        <v>-197.2040399963216</v>
       </c>
       <c r="D473" t="n">
         <v>361</v>
@@ -13148,10 +13148,10 @@
         <v>-315.4040399963221</v>
       </c>
       <c r="F473" t="n">
-        <v>-538.0000000000001</v>
+        <v>-683.5000000000001</v>
       </c>
       <c r="G473" t="n">
-        <v>-635.7488570093457</v>
+        <v>-781.2488570093456</v>
       </c>
       <c r="H473" t="n">
         <v>-824</v>
@@ -13162,10 +13162,10 @@
         <v>46220</v>
       </c>
       <c r="B474" t="n">
-        <v>237.1000000000001</v>
+        <v>91.60000000000002</v>
       </c>
       <c r="C474" t="n">
-        <v>-76.10403999632172</v>
+        <v>-221.6040399963216</v>
       </c>
       <c r="D474" t="n">
         <v>333</v>
@@ -13174,10 +13174,10 @@
         <v>-313.2040399963221</v>
       </c>
       <c r="F474" t="n">
-        <v>-564.6000000000001</v>
+        <v>-710.1000000000001</v>
       </c>
       <c r="G474" t="n">
-        <v>-660.1488570093456</v>
+        <v>-805.6488570093455</v>
       </c>
       <c r="H474" t="n">
         <v>-852</v>
@@ -13188,10 +13188,10 @@
         <v>46221</v>
       </c>
       <c r="B475" t="n">
-        <v>237.1000000000001</v>
+        <v>91.60000000000002</v>
       </c>
       <c r="C475" t="n">
-        <v>-76.10403999632172</v>
+        <v>-221.6040399963216</v>
       </c>
       <c r="D475" t="n">
         <v>333</v>
@@ -13200,10 +13200,10 @@
         <v>-313.2040399963221</v>
       </c>
       <c r="F475" t="n">
-        <v>-564.6000000000001</v>
+        <v>-710.1000000000001</v>
       </c>
       <c r="G475" t="n">
-        <v>-660.1488570093456</v>
+        <v>-805.6488570093455</v>
       </c>
       <c r="H475" t="n">
         <v>-852</v>
@@ -13214,10 +13214,10 @@
         <v>46222</v>
       </c>
       <c r="B476" t="n">
-        <v>237.1000000000001</v>
+        <v>91.60000000000002</v>
       </c>
       <c r="C476" t="n">
-        <v>-76.10403999632172</v>
+        <v>-221.6040399963216</v>
       </c>
       <c r="D476" t="n">
         <v>333</v>
@@ -13226,10 +13226,10 @@
         <v>-313.2040399963221</v>
       </c>
       <c r="F476" t="n">
-        <v>-564.6000000000001</v>
+        <v>-710.1000000000001</v>
       </c>
       <c r="G476" t="n">
-        <v>-660.1488570093456</v>
+        <v>-805.6488570093455</v>
       </c>
       <c r="H476" t="n">
         <v>-852</v>
@@ -13240,10 +13240,10 @@
         <v>46223</v>
       </c>
       <c r="B477" t="n">
-        <v>248.8</v>
+        <v>103.3</v>
       </c>
       <c r="C477" t="n">
-        <v>-69.39403999632172</v>
+        <v>-214.8940399963216</v>
       </c>
       <c r="D477" t="n">
         <v>344</v>
@@ -13252,10 +13252,10 @@
         <v>-318.1940399963221</v>
       </c>
       <c r="F477" t="n">
-        <v>-552.9000000000001</v>
+        <v>-698.4000000000001</v>
       </c>
       <c r="G477" t="n">
-        <v>-653.4388570093456</v>
+        <v>-798.9388570093455</v>
       </c>
       <c r="H477" t="n">
         <v>-841</v>
@@ -13266,10 +13266,10 @@
         <v>46224</v>
       </c>
       <c r="B478" t="n">
-        <v>227.3</v>
+        <v>81.80000000000003</v>
       </c>
       <c r="C478" t="n">
-        <v>-96.86403999632172</v>
+        <v>-242.3640399963216</v>
       </c>
       <c r="D478" t="n">
         <v>335</v>
@@ -13278,10 +13278,10 @@
         <v>-324.1640399963222</v>
       </c>
       <c r="F478" t="n">
-        <v>-574.4000000000001</v>
+        <v>-719.9000000000001</v>
       </c>
       <c r="G478" t="n">
-        <v>-680.9088570093456</v>
+        <v>-826.4088570093455</v>
       </c>
       <c r="H478" t="n">
         <v>-850</v>
@@ -13292,10 +13292,10 @@
         <v>46225</v>
       </c>
       <c r="B479" t="n">
-        <v>227.3</v>
+        <v>81.80000000000003</v>
       </c>
       <c r="C479" t="n">
-        <v>-99.61403999632172</v>
+        <v>-245.1140399963216</v>
       </c>
       <c r="D479" t="n">
         <v>335</v>
@@ -13304,10 +13304,10 @@
         <v>-326.9140399963222</v>
       </c>
       <c r="F479" t="n">
-        <v>-574.4000000000001</v>
+        <v>-719.9000000000001</v>
       </c>
       <c r="G479" t="n">
-        <v>-683.6588570093456</v>
+        <v>-829.1588570093455</v>
       </c>
       <c r="H479" t="n">
         <v>-850</v>
@@ -13318,10 +13318,10 @@
         <v>46226</v>
       </c>
       <c r="B480" t="n">
-        <v>227.3</v>
+        <v>81.80000000000003</v>
       </c>
       <c r="C480" t="n">
-        <v>-103.3340399963217</v>
+        <v>-248.8340399963216</v>
       </c>
       <c r="D480" t="n">
         <v>335</v>
@@ -13330,10 +13330,10 @@
         <v>-330.6340399963222</v>
       </c>
       <c r="F480" t="n">
-        <v>-574.4000000000001</v>
+        <v>-719.9000000000001</v>
       </c>
       <c r="G480" t="n">
-        <v>-687.3788570093457</v>
+        <v>-832.8788570093454</v>
       </c>
       <c r="H480" t="n">
         <v>-850</v>
@@ -13344,10 +13344,10 @@
         <v>46227</v>
       </c>
       <c r="B481" t="n">
-        <v>227.3</v>
+        <v>81.80000000000003</v>
       </c>
       <c r="C481" t="n">
-        <v>-106.4840399963217</v>
+        <v>-251.9840399963216</v>
       </c>
       <c r="D481" t="n">
         <v>335</v>
@@ -13356,10 +13356,10 @@
         <v>-333.7840399963222</v>
       </c>
       <c r="F481" t="n">
-        <v>-574.4000000000001</v>
+        <v>-719.9000000000001</v>
       </c>
       <c r="G481" t="n">
-        <v>-690.5288570093456</v>
+        <v>-836.0288570093455</v>
       </c>
       <c r="H481" t="n">
         <v>-850</v>
@@ -13370,10 +13370,10 @@
         <v>46228</v>
       </c>
       <c r="B482" t="n">
-        <v>227.3</v>
+        <v>81.80000000000003</v>
       </c>
       <c r="C482" t="n">
-        <v>-106.4840399963217</v>
+        <v>-251.9840399963216</v>
       </c>
       <c r="D482" t="n">
         <v>335</v>
@@ -13382,10 +13382,10 @@
         <v>-333.7840399963222</v>
       </c>
       <c r="F482" t="n">
-        <v>-574.4000000000001</v>
+        <v>-719.9000000000001</v>
       </c>
       <c r="G482" t="n">
-        <v>-690.5288570093456</v>
+        <v>-836.0288570093455</v>
       </c>
       <c r="H482" t="n">
         <v>-850</v>
@@ -13396,10 +13396,10 @@
         <v>46229</v>
       </c>
       <c r="B483" t="n">
-        <v>227.3</v>
+        <v>81.80000000000003</v>
       </c>
       <c r="C483" t="n">
-        <v>-106.4840399963217</v>
+        <v>-251.9840399963216</v>
       </c>
       <c r="D483" t="n">
         <v>335</v>
@@ -13408,10 +13408,10 @@
         <v>-333.7840399963222</v>
       </c>
       <c r="F483" t="n">
-        <v>-574.4000000000001</v>
+        <v>-719.9000000000001</v>
       </c>
       <c r="G483" t="n">
-        <v>-690.5288570093456</v>
+        <v>-836.0288570093455</v>
       </c>
       <c r="H483" t="n">
         <v>-850</v>
@@ -13422,10 +13422,10 @@
         <v>46230</v>
       </c>
       <c r="B484" t="n">
-        <v>345.9</v>
+        <v>200.4</v>
       </c>
       <c r="C484" t="n">
-        <v>4.265960003678288</v>
+        <v>-141.2340399963215</v>
       </c>
       <c r="D484" t="n">
         <v>435</v>
@@ -13434,10 +13434,10 @@
         <v>-341.6340399963222</v>
       </c>
       <c r="F484" t="n">
-        <v>-455.8000000000001</v>
+        <v>-601.3000000000002</v>
       </c>
       <c r="G484" t="n">
-        <v>-579.7788570093456</v>
+        <v>-725.2788570093455</v>
       </c>
       <c r="H484" t="n">
         <v>-750</v>
@@ -13448,10 +13448,10 @@
         <v>46231</v>
       </c>
       <c r="B485" t="n">
-        <v>345.9</v>
+        <v>200.4</v>
       </c>
       <c r="C485" t="n">
-        <v>1.275960003678287</v>
+        <v>-144.2240399963216</v>
       </c>
       <c r="D485" t="n">
         <v>454</v>
@@ -13460,10 +13460,10 @@
         <v>-344.6240399963222</v>
       </c>
       <c r="F485" t="n">
-        <v>-455.8000000000001</v>
+        <v>-601.3000000000002</v>
       </c>
       <c r="G485" t="n">
-        <v>-582.7688570093457</v>
+        <v>-728.2688570093455</v>
       </c>
       <c r="H485" t="n">
         <v>-731</v>
@@ -13474,10 +13474,10 @@
         <v>46232</v>
       </c>
       <c r="B486" t="n">
-        <v>345.9</v>
+        <v>200.4</v>
       </c>
       <c r="C486" t="n">
-        <v>-2.684039996321713</v>
+        <v>-148.1840399963216</v>
       </c>
       <c r="D486" t="n">
         <v>454</v>
@@ -13486,10 +13486,10 @@
         <v>-348.5840399963222</v>
       </c>
       <c r="F486" t="n">
-        <v>-455.8000000000001</v>
+        <v>-601.3000000000002</v>
       </c>
       <c r="G486" t="n">
-        <v>-586.7288570093457</v>
+        <v>-732.2288570093455</v>
       </c>
       <c r="H486" t="n">
         <v>-731</v>
@@ -13500,10 +13500,10 @@
         <v>46233</v>
       </c>
       <c r="B487" t="n">
-        <v>345.9</v>
+        <v>200.4</v>
       </c>
       <c r="C487" t="n">
-        <v>-8.244039996321712</v>
+        <v>-153.7440399963216</v>
       </c>
       <c r="D487" t="n">
         <v>454</v>
@@ -13512,10 +13512,10 @@
         <v>-354.1440399963222</v>
       </c>
       <c r="F487" t="n">
-        <v>-455.8000000000001</v>
+        <v>-601.3000000000002</v>
       </c>
       <c r="G487" t="n">
-        <v>-592.2888570093456</v>
+        <v>-737.7888570093455</v>
       </c>
       <c r="H487" t="n">
         <v>-731</v>
@@ -13526,10 +13526,10 @@
         <v>46234</v>
       </c>
       <c r="B488" t="n">
-        <v>345.9</v>
+        <v>200.4</v>
       </c>
       <c r="C488" t="n">
-        <v>-11.24403999632171</v>
+        <v>-156.7440399963216</v>
       </c>
       <c r="D488" t="n">
         <v>454</v>
@@ -13538,10 +13538,10 @@
         <v>-357.1440399963222</v>
       </c>
       <c r="F488" t="n">
-        <v>-455.8000000000001</v>
+        <v>-601.3000000000002</v>
       </c>
       <c r="G488" t="n">
-        <v>-595.2888570093456</v>
+        <v>-740.7888570093455</v>
       </c>
       <c r="H488" t="n">
         <v>-731</v>
@@ -13552,10 +13552,10 @@
         <v>46235</v>
       </c>
       <c r="B489" t="n">
-        <v>345.9</v>
+        <v>200.4</v>
       </c>
       <c r="C489" t="n">
-        <v>-11.24403999632171</v>
+        <v>-156.7440399963216</v>
       </c>
       <c r="D489" t="n">
         <v>454</v>
@@ -13564,10 +13564,10 @@
         <v>-357.1440399963222</v>
       </c>
       <c r="F489" t="n">
-        <v>-455.8000000000001</v>
+        <v>-601.3000000000002</v>
       </c>
       <c r="G489" t="n">
-        <v>-595.2888570093456</v>
+        <v>-740.7888570093455</v>
       </c>
       <c r="H489" t="n">
         <v>-731</v>
@@ -13578,10 +13578,10 @@
         <v>46236</v>
       </c>
       <c r="B490" t="n">
-        <v>345.9</v>
+        <v>200.4</v>
       </c>
       <c r="C490" t="n">
-        <v>-11.24403999632171</v>
+        <v>-156.7440399963216</v>
       </c>
       <c r="D490" t="n">
         <v>454</v>
@@ -13590,10 +13590,10 @@
         <v>-357.1440399963222</v>
       </c>
       <c r="F490" t="n">
-        <v>-455.8000000000001</v>
+        <v>-601.3000000000002</v>
       </c>
       <c r="G490" t="n">
-        <v>-595.2888570093456</v>
+        <v>-740.7888570093455</v>
       </c>
       <c r="H490" t="n">
         <v>-731</v>
@@ -13604,10 +13604,10 @@
         <v>46237</v>
       </c>
       <c r="B491" t="n">
-        <v>345.9</v>
+        <v>200.4</v>
       </c>
       <c r="C491" t="n">
-        <v>-13.68403999632171</v>
+        <v>-159.1840399963216</v>
       </c>
       <c r="D491" t="n">
         <v>454</v>
@@ -13616,10 +13616,10 @@
         <v>-359.5840399963222</v>
       </c>
       <c r="F491" t="n">
-        <v>-455.8000000000001</v>
+        <v>-601.3000000000002</v>
       </c>
       <c r="G491" t="n">
-        <v>-597.7288570093457</v>
+        <v>-743.2288570093455</v>
       </c>
       <c r="H491" t="n">
         <v>-731</v>
@@ -13630,10 +13630,10 @@
         <v>46238</v>
       </c>
       <c r="B492" t="n">
-        <v>387.3000000000001</v>
+        <v>241.8</v>
       </c>
       <c r="C492" t="n">
-        <v>25.53596000367829</v>
+        <v>-119.9640399963216</v>
       </c>
       <c r="D492" t="n">
         <v>496</v>
@@ -13642,10 +13642,10 @@
         <v>-361.7640399963222</v>
       </c>
       <c r="F492" t="n">
-        <v>-414.4000000000001</v>
+        <v>-559.9000000000001</v>
       </c>
       <c r="G492" t="n">
-        <v>-558.5088570093457</v>
+        <v>-704.0088570093455</v>
       </c>
       <c r="H492" t="n">
         <v>-689</v>
@@ -13656,10 +13656,10 @@
         <v>46239</v>
       </c>
       <c r="B493" t="n">
-        <v>387.3000000000001</v>
+        <v>241.8</v>
       </c>
       <c r="C493" t="n">
-        <v>21.34596000367829</v>
+        <v>-124.1540399963216</v>
       </c>
       <c r="D493" t="n">
         <v>496</v>
@@ -13668,10 +13668,10 @@
         <v>-365.9540399963222</v>
       </c>
       <c r="F493" t="n">
-        <v>-414.4000000000001</v>
+        <v>-559.9000000000001</v>
       </c>
       <c r="G493" t="n">
-        <v>-562.6988570093456</v>
+        <v>-708.1988570093455</v>
       </c>
       <c r="H493" t="n">
         <v>-689</v>
@@ -13682,10 +13682,10 @@
         <v>46240</v>
       </c>
       <c r="B494" t="n">
-        <v>387.3000000000001</v>
+        <v>241.8</v>
       </c>
       <c r="C494" t="n">
-        <v>20.38596000367829</v>
+        <v>-125.1140399963216</v>
       </c>
       <c r="D494" t="n">
         <v>496</v>
@@ -13694,10 +13694,10 @@
         <v>-366.9140399963222</v>
       </c>
       <c r="F494" t="n">
-        <v>-414.4000000000001</v>
+        <v>-559.9000000000001</v>
       </c>
       <c r="G494" t="n">
-        <v>-563.6588570093456</v>
+        <v>-709.1588570093455</v>
       </c>
       <c r="H494" t="n">
         <v>-689</v>
@@ -13708,10 +13708,10 @@
         <v>46241</v>
       </c>
       <c r="B495" t="n">
-        <v>387.3000000000001</v>
+        <v>241.8</v>
       </c>
       <c r="C495" t="n">
-        <v>20.58596000367829</v>
+        <v>-124.9140399963215</v>
       </c>
       <c r="D495" t="n">
         <v>496</v>
@@ -13720,10 +13720,10 @@
         <v>-366.7140399963222</v>
       </c>
       <c r="F495" t="n">
-        <v>-414.4000000000001</v>
+        <v>-559.9000000000001</v>
       </c>
       <c r="G495" t="n">
-        <v>-563.4588570093456</v>
+        <v>-708.9588570093455</v>
       </c>
       <c r="H495" t="n">
         <v>-689</v>
@@ -13734,10 +13734,10 @@
         <v>46242</v>
       </c>
       <c r="B496" t="n">
-        <v>387.3000000000001</v>
+        <v>241.8</v>
       </c>
       <c r="C496" t="n">
-        <v>20.58596000367829</v>
+        <v>-124.9140399963215</v>
       </c>
       <c r="D496" t="n">
         <v>496</v>
@@ -13746,10 +13746,10 @@
         <v>-366.7140399963222</v>
       </c>
       <c r="F496" t="n">
-        <v>-414.4000000000001</v>
+        <v>-559.9000000000001</v>
       </c>
       <c r="G496" t="n">
-        <v>-563.4588570093456</v>
+        <v>-708.9588570093455</v>
       </c>
       <c r="H496" t="n">
         <v>-689</v>
@@ -13760,10 +13760,10 @@
         <v>46243</v>
       </c>
       <c r="B497" t="n">
-        <v>387.3000000000001</v>
+        <v>241.8</v>
       </c>
       <c r="C497" t="n">
-        <v>20.58596000367829</v>
+        <v>-124.9140399963215</v>
       </c>
       <c r="D497" t="n">
         <v>496</v>
@@ -13772,10 +13772,10 @@
         <v>-366.7140399963222</v>
       </c>
       <c r="F497" t="n">
-        <v>-414.4000000000001</v>
+        <v>-559.9000000000001</v>
       </c>
       <c r="G497" t="n">
-        <v>-563.4588570093456</v>
+        <v>-708.9588570093455</v>
       </c>
       <c r="H497" t="n">
         <v>-689</v>
@@ -13786,10 +13786,10 @@
         <v>46244</v>
       </c>
       <c r="B498" t="n">
-        <v>482.7</v>
+        <v>337.2</v>
       </c>
       <c r="C498" t="n">
-        <v>115.6359600036783</v>
+        <v>-29.86403999632154</v>
       </c>
       <c r="D498" t="n">
         <v>591</v>
@@ -13798,10 +13798,10 @@
         <v>-367.0640399963222</v>
       </c>
       <c r="F498" t="n">
-        <v>-319.0000000000001</v>
+        <v>-464.5000000000001</v>
       </c>
       <c r="G498" t="n">
-        <v>-468.4088570093456</v>
+        <v>-613.9088570093454</v>
       </c>
       <c r="H498" t="n">
         <v>-594</v>
@@ -13812,10 +13812,10 @@
         <v>46245</v>
       </c>
       <c r="B499" t="n">
-        <v>482.7</v>
+        <v>337.2</v>
       </c>
       <c r="C499" t="n">
-        <v>115.6359600036783</v>
+        <v>-29.86403999632154</v>
       </c>
       <c r="D499" t="n">
         <v>636</v>
@@ -13824,10 +13824,10 @@
         <v>-367.0640399963222</v>
       </c>
       <c r="F499" t="n">
-        <v>-319.0000000000001</v>
+        <v>-464.5000000000001</v>
       </c>
       <c r="G499" t="n">
-        <v>-468.4088570093456</v>
+        <v>-613.9088570093454</v>
       </c>
       <c r="H499" t="n">
         <v>-549</v>
@@ -13838,10 +13838,10 @@
         <v>46246</v>
       </c>
       <c r="B500" t="n">
-        <v>482.7</v>
+        <v>337.2</v>
       </c>
       <c r="C500" t="n">
-        <v>114.1359600036783</v>
+        <v>-31.36403999632154</v>
       </c>
       <c r="D500" t="n">
         <v>636</v>
@@ -13850,10 +13850,10 @@
         <v>-368.5640399963222</v>
       </c>
       <c r="F500" t="n">
-        <v>-319.0000000000001</v>
+        <v>-464.5000000000001</v>
       </c>
       <c r="G500" t="n">
-        <v>-469.9088570093456</v>
+        <v>-615.4088570093454</v>
       </c>
       <c r="H500" t="n">
         <v>-549</v>
@@ -13864,10 +13864,10 @@
         <v>46247</v>
       </c>
       <c r="B501" t="n">
-        <v>482.7</v>
+        <v>337.2</v>
       </c>
       <c r="C501" t="n">
-        <v>113.3359600036783</v>
+        <v>-32.16403999632153</v>
       </c>
       <c r="D501" t="n">
         <v>636</v>
@@ -13876,10 +13876,10 @@
         <v>-369.3640399963222</v>
       </c>
       <c r="F501" t="n">
-        <v>-319.0000000000001</v>
+        <v>-464.5000000000001</v>
       </c>
       <c r="G501" t="n">
-        <v>-470.7088570093456</v>
+        <v>-616.2088570093455</v>
       </c>
       <c r="H501" t="n">
         <v>-549</v>
@@ -13890,10 +13890,10 @@
         <v>46248</v>
       </c>
       <c r="B502" t="n">
-        <v>482.7</v>
+        <v>337.2</v>
       </c>
       <c r="C502" t="n">
-        <v>111.8559600036783</v>
+        <v>-33.64403999632153</v>
       </c>
       <c r="D502" t="n">
         <v>636</v>
@@ -13902,10 +13902,10 @@
         <v>-370.8440399963222</v>
       </c>
       <c r="F502" t="n">
-        <v>-319.0000000000001</v>
+        <v>-464.5000000000001</v>
       </c>
       <c r="G502" t="n">
-        <v>-472.1888570093456</v>
+        <v>-617.6888570093455</v>
       </c>
       <c r="H502" t="n">
         <v>-549</v>
@@ -13916,10 +13916,10 @@
         <v>46249</v>
       </c>
       <c r="B503" t="n">
-        <v>482.7</v>
+        <v>337.2</v>
       </c>
       <c r="C503" t="n">
-        <v>111.8559600036783</v>
+        <v>-33.64403999632153</v>
       </c>
       <c r="D503" t="n">
         <v>636</v>
@@ -13928,10 +13928,10 @@
         <v>-370.8440399963222</v>
       </c>
       <c r="F503" t="n">
-        <v>-319.0000000000001</v>
+        <v>-464.5000000000001</v>
       </c>
       <c r="G503" t="n">
-        <v>-472.1888570093456</v>
+        <v>-617.6888570093455</v>
       </c>
       <c r="H503" t="n">
         <v>-549</v>
@@ -13942,10 +13942,10 @@
         <v>46250</v>
       </c>
       <c r="B504" t="n">
-        <v>482.7</v>
+        <v>337.2</v>
       </c>
       <c r="C504" t="n">
-        <v>111.8559600036783</v>
+        <v>-33.64403999632153</v>
       </c>
       <c r="D504" t="n">
         <v>636</v>
@@ -13954,10 +13954,10 @@
         <v>-370.8440399963222</v>
       </c>
       <c r="F504" t="n">
-        <v>-319.0000000000001</v>
+        <v>-464.5000000000001</v>
       </c>
       <c r="G504" t="n">
-        <v>-472.1888570093456</v>
+        <v>-617.6888570093455</v>
       </c>
       <c r="H504" t="n">
         <v>-549</v>
@@ -13968,10 +13968,10 @@
         <v>46251</v>
       </c>
       <c r="B505" t="n">
-        <v>482.7</v>
+        <v>337.2</v>
       </c>
       <c r="C505" t="n">
-        <v>108.7559600036783</v>
+        <v>-36.74403999632153</v>
       </c>
       <c r="D505" t="n">
         <v>636</v>
@@ -13980,10 +13980,10 @@
         <v>-373.9440399963223</v>
       </c>
       <c r="F505" t="n">
-        <v>-319.0000000000001</v>
+        <v>-464.5000000000001</v>
       </c>
       <c r="G505" t="n">
-        <v>-475.2888570093456</v>
+        <v>-620.7888570093455</v>
       </c>
       <c r="H505" t="n">
         <v>-549</v>
@@ -13994,10 +13994,10 @@
         <v>46252</v>
       </c>
       <c r="B506" t="n">
-        <v>653.8000000000001</v>
+        <v>508.3000000000001</v>
       </c>
       <c r="C506" t="n">
-        <v>276.0059600036783</v>
+        <v>130.5059600036785</v>
       </c>
       <c r="D506" t="n">
         <v>808</v>
@@ -14006,10 +14006,10 @@
         <v>-377.7940399963223</v>
       </c>
       <c r="F506" t="n">
-        <v>-147.9000000000001</v>
+        <v>-293.4000000000001</v>
       </c>
       <c r="G506" t="n">
-        <v>-308.0388570093456</v>
+        <v>-453.5388570093455</v>
       </c>
       <c r="H506" t="n">
         <v>-377</v>
@@ -14020,10 +14020,10 @@
         <v>46253</v>
       </c>
       <c r="B507" t="n">
-        <v>653.8000000000001</v>
+        <v>508.3000000000001</v>
       </c>
       <c r="C507" t="n">
-        <v>270.4259600036783</v>
+        <v>124.9259600036785</v>
       </c>
       <c r="D507" t="n">
         <v>808</v>
@@ -14032,10 +14032,10 @@
         <v>-383.3740399963223</v>
       </c>
       <c r="F507" t="n">
-        <v>-147.9000000000001</v>
+        <v>-293.4000000000001</v>
       </c>
       <c r="G507" t="n">
-        <v>-313.6188570093456</v>
+        <v>-459.1188570093454</v>
       </c>
       <c r="H507" t="n">
         <v>-377</v>
@@ -14046,10 +14046,10 @@
         <v>46254</v>
       </c>
       <c r="B508" t="n">
-        <v>653.5000000000001</v>
+        <v>508.0000000000001</v>
       </c>
       <c r="C508" t="n">
-        <v>267.9259600036783</v>
+        <v>122.4259600036785</v>
       </c>
       <c r="D508" t="n">
         <v>809</v>
@@ -14058,10 +14058,10 @@
         <v>-385.5740399963223</v>
       </c>
       <c r="F508" t="n">
-        <v>-148.2</v>
+        <v>-293.7000000000001</v>
       </c>
       <c r="G508" t="n">
-        <v>-316.1188570093456</v>
+        <v>-461.6188570093454</v>
       </c>
       <c r="H508" t="n">
         <v>-376</v>
@@ -14072,10 +14072,10 @@
         <v>46255</v>
       </c>
       <c r="B509" t="n">
-        <v>653.5000000000001</v>
+        <v>508.0000000000001</v>
       </c>
       <c r="C509" t="n">
-        <v>267.9259600036783</v>
+        <v>122.4259600036785</v>
       </c>
       <c r="D509" t="n">
         <v>809</v>
@@ -14084,10 +14084,10 @@
         <v>-385.5740399963223</v>
       </c>
       <c r="F509" t="n">
-        <v>-148.2</v>
+        <v>-293.7000000000001</v>
       </c>
       <c r="G509" t="n">
-        <v>-316.1188570093456</v>
+        <v>-461.6188570093454</v>
       </c>
       <c r="H509" t="n">
         <v>-376</v>
@@ -14098,10 +14098,10 @@
         <v>46256</v>
       </c>
       <c r="B510" t="n">
-        <v>653.5000000000001</v>
+        <v>508.0000000000001</v>
       </c>
       <c r="C510" t="n">
-        <v>267.9259600036783</v>
+        <v>122.4259600036785</v>
       </c>
       <c r="D510" t="n">
         <v>809</v>
@@ -14110,10 +14110,10 @@
         <v>-385.5740399963223</v>
       </c>
       <c r="F510" t="n">
-        <v>-148.2</v>
+        <v>-293.7000000000001</v>
       </c>
       <c r="G510" t="n">
-        <v>-316.1188570093456</v>
+        <v>-461.6188570093454</v>
       </c>
       <c r="H510" t="n">
         <v>-376</v>
@@ -14124,10 +14124,10 @@
         <v>46257</v>
       </c>
       <c r="B511" t="n">
-        <v>653.5000000000001</v>
+        <v>508.0000000000001</v>
       </c>
       <c r="C511" t="n">
-        <v>267.9259600036783</v>
+        <v>122.4259600036785</v>
       </c>
       <c r="D511" t="n">
         <v>809</v>
@@ -14136,10 +14136,10 @@
         <v>-385.5740399963223</v>
       </c>
       <c r="F511" t="n">
-        <v>-148.2</v>
+        <v>-293.7000000000001</v>
       </c>
       <c r="G511" t="n">
-        <v>-316.1188570093456</v>
+        <v>-461.6188570093454</v>
       </c>
       <c r="H511" t="n">
         <v>-376</v>
@@ -14150,10 +14150,10 @@
         <v>46258</v>
       </c>
       <c r="B512" t="n">
-        <v>653.5000000000001</v>
+        <v>508.0000000000001</v>
       </c>
       <c r="C512" t="n">
-        <v>267.9259600036783</v>
+        <v>122.4259600036785</v>
       </c>
       <c r="D512" t="n">
         <v>809</v>
@@ -14162,10 +14162,10 @@
         <v>-385.5740399963223</v>
       </c>
       <c r="F512" t="n">
-        <v>-148.2</v>
+        <v>-293.7000000000001</v>
       </c>
       <c r="G512" t="n">
-        <v>-316.1188570093456</v>
+        <v>-461.6188570093454</v>
       </c>
       <c r="H512" t="n">
         <v>-376</v>
@@ -14176,10 +14176,10 @@
         <v>46259</v>
       </c>
       <c r="B513" t="n">
-        <v>664.8000000000001</v>
+        <v>519.3000000000001</v>
       </c>
       <c r="C513" t="n">
-        <v>276.4059600036783</v>
+        <v>130.9059600036785</v>
       </c>
       <c r="D513" t="n">
         <v>816</v>
@@ -14188,10 +14188,10 @@
         <v>-388.3940399963222</v>
       </c>
       <c r="F513" t="n">
-        <v>-136.9000000000001</v>
+        <v>-282.4000000000001</v>
       </c>
       <c r="G513" t="n">
-        <v>-307.6388570093456</v>
+        <v>-453.1388570093454</v>
       </c>
       <c r="H513" t="n">
         <v>-369</v>
@@ -14202,10 +14202,10 @@
         <v>46260</v>
       </c>
       <c r="B514" t="n">
-        <v>653.9000000000001</v>
+        <v>508.4000000000001</v>
       </c>
       <c r="C514" t="n">
-        <v>261.3859600036783</v>
+        <v>115.8859600036785</v>
       </c>
       <c r="D514" t="n">
         <v>813</v>
@@ -14214,10 +14214,10 @@
         <v>-392.5140399963223</v>
       </c>
       <c r="F514" t="n">
-        <v>-147.8000000000001</v>
+        <v>-293.3000000000001</v>
       </c>
       <c r="G514" t="n">
-        <v>-322.6588570093456</v>
+        <v>-468.1588570093455</v>
       </c>
       <c r="H514" t="n">
         <v>-372</v>
@@ -14228,10 +14228,10 @@
         <v>46261</v>
       </c>
       <c r="B515" t="n">
-        <v>653.9000000000001</v>
+        <v>508.4000000000001</v>
       </c>
       <c r="C515" t="n">
-        <v>261.3859600036783</v>
+        <v>115.8859600036785</v>
       </c>
       <c r="D515" t="n">
         <v>813</v>
@@ -14240,10 +14240,10 @@
         <v>-392.5140399963223</v>
       </c>
       <c r="F515" t="n">
-        <v>-147.8000000000001</v>
+        <v>-293.3000000000001</v>
       </c>
       <c r="G515" t="n">
-        <v>-322.6588570093456</v>
+        <v>-468.1588570093455</v>
       </c>
       <c r="H515" t="n">
         <v>-372</v>
@@ -14254,10 +14254,10 @@
         <v>46262</v>
       </c>
       <c r="B516" t="n">
-        <v>653.9000000000001</v>
+        <v>508.4000000000001</v>
       </c>
       <c r="C516" t="n">
-        <v>261.4859600036784</v>
+        <v>115.9859600036785</v>
       </c>
       <c r="D516" t="n">
         <v>813</v>
@@ -14266,10 +14266,10 @@
         <v>-392.4140399963222</v>
       </c>
       <c r="F516" t="n">
-        <v>-147.8000000000001</v>
+        <v>-293.3000000000001</v>
       </c>
       <c r="G516" t="n">
-        <v>-322.5588570093456</v>
+        <v>-468.0588570093454</v>
       </c>
       <c r="H516" t="n">
         <v>-372</v>
@@ -14280,10 +14280,10 @@
         <v>46263</v>
       </c>
       <c r="B517" t="n">
-        <v>653.9000000000001</v>
+        <v>508.4000000000001</v>
       </c>
       <c r="C517" t="n">
-        <v>261.4859600036784</v>
+        <v>115.9859600036785</v>
       </c>
       <c r="D517" t="n">
         <v>813</v>
@@ -14292,10 +14292,10 @@
         <v>-392.4140399963222</v>
       </c>
       <c r="F517" t="n">
-        <v>-147.8000000000001</v>
+        <v>-293.3000000000001</v>
       </c>
       <c r="G517" t="n">
-        <v>-322.5588570093456</v>
+        <v>-468.0588570093454</v>
       </c>
       <c r="H517" t="n">
         <v>-372</v>
@@ -14306,10 +14306,10 @@
         <v>46264</v>
       </c>
       <c r="B518" t="n">
-        <v>653.9000000000001</v>
+        <v>508.4000000000001</v>
       </c>
       <c r="C518" t="n">
-        <v>261.4859600036784</v>
+        <v>115.9859600036785</v>
       </c>
       <c r="D518" t="n">
         <v>813</v>
@@ -14318,10 +14318,10 @@
         <v>-392.4140399963222</v>
       </c>
       <c r="F518" t="n">
-        <v>-147.8000000000001</v>
+        <v>-293.3000000000001</v>
       </c>
       <c r="G518" t="n">
-        <v>-322.5588570093456</v>
+        <v>-468.0588570093454</v>
       </c>
       <c r="H518" t="n">
         <v>-372</v>
@@ -14332,10 +14332,10 @@
         <v>46265</v>
       </c>
       <c r="B519" t="n">
-        <v>745.3000000000001</v>
+        <v>599.8000000000001</v>
       </c>
       <c r="C519" t="n">
-        <v>343.0859600036784</v>
+        <v>197.5859600036785</v>
       </c>
       <c r="D519" t="n">
         <v>813</v>
@@ -14344,10 +14344,10 @@
         <v>-402.2140399963222</v>
       </c>
       <c r="F519" t="n">
-        <v>-56.40000000000009</v>
+        <v>-201.9000000000001</v>
       </c>
       <c r="G519" t="n">
-        <v>-240.9588570093455</v>
+        <v>-386.4588570093455</v>
       </c>
       <c r="H519" t="n">
         <v>-372</v>
@@ -14358,10 +14358,10 @@
         <v>46266</v>
       </c>
       <c r="B520" t="n">
-        <v>689.6</v>
+        <v>544.1</v>
       </c>
       <c r="C520" t="n">
-        <v>283.0859600036784</v>
+        <v>137.5859600036785</v>
       </c>
       <c r="D520" t="n">
         <v>849</v>
@@ -14370,10 +14370,10 @@
         <v>-406.5140399963223</v>
       </c>
       <c r="F520" t="n">
-        <v>-112.1000000000001</v>
+        <v>-257.6000000000001</v>
       </c>
       <c r="G520" t="n">
-        <v>-300.9588570093455</v>
+        <v>-446.4588570093455</v>
       </c>
       <c r="H520" t="n">
         <v>-336</v>
@@ -14384,10 +14384,10 @@
         <v>46267</v>
       </c>
       <c r="B521" t="n">
-        <v>689.6</v>
+        <v>544.1</v>
       </c>
       <c r="C521" t="n">
-        <v>278.3859600036784</v>
+        <v>132.8859600036785</v>
       </c>
       <c r="D521" t="n">
         <v>849</v>
@@ -14396,10 +14396,10 @@
         <v>-411.2140399963222</v>
       </c>
       <c r="F521" t="n">
-        <v>-112.1000000000001</v>
+        <v>-257.6000000000001</v>
       </c>
       <c r="G521" t="n">
-        <v>-305.6588570093455</v>
+        <v>-451.1588570093454</v>
       </c>
       <c r="H521" t="n">
         <v>-336</v>
@@ -14410,10 +14410,10 @@
         <v>46268</v>
       </c>
       <c r="B522" t="n">
-        <v>689.6</v>
+        <v>544.1</v>
       </c>
       <c r="C522" t="n">
-        <v>277.0859600036784</v>
+        <v>131.5859600036785</v>
       </c>
       <c r="D522" t="n">
         <v>849</v>
@@ -14422,10 +14422,10 @@
         <v>-412.5140399963223</v>
       </c>
       <c r="F522" t="n">
-        <v>-112.1000000000001</v>
+        <v>-257.6000000000001</v>
       </c>
       <c r="G522" t="n">
-        <v>-306.9588570093455</v>
+        <v>-452.4588570093455</v>
       </c>
       <c r="H522" t="n">
         <v>-336</v>
@@ -14436,10 +14436,10 @@
         <v>46269</v>
       </c>
       <c r="B523" t="n">
-        <v>715.7</v>
+        <v>570.2</v>
       </c>
       <c r="C523" t="n">
-        <v>301.0859600036784</v>
+        <v>155.5859600036785</v>
       </c>
       <c r="D523" t="n">
         <v>876</v>
@@ -14448,10 +14448,10 @@
         <v>-414.6140399963223</v>
       </c>
       <c r="F523" t="n">
-        <v>-86.00000000000011</v>
+        <v>-231.5000000000001</v>
       </c>
       <c r="G523" t="n">
-        <v>-282.9588570093455</v>
+        <v>-428.4588570093455</v>
       </c>
       <c r="H523" t="n">
         <v>-309</v>
@@ -14462,10 +14462,10 @@
         <v>46270</v>
       </c>
       <c r="B524" t="n">
-        <v>715.7</v>
+        <v>570.2</v>
       </c>
       <c r="C524" t="n">
-        <v>301.0859600036784</v>
+        <v>155.5859600036785</v>
       </c>
       <c r="D524" t="n">
         <v>876</v>
@@ -14474,10 +14474,10 @@
         <v>-414.6140399963223</v>
       </c>
       <c r="F524" t="n">
-        <v>-86.00000000000011</v>
+        <v>-231.5000000000001</v>
       </c>
       <c r="G524" t="n">
-        <v>-282.9588570093455</v>
+        <v>-428.4588570093455</v>
       </c>
       <c r="H524" t="n">
         <v>-309</v>
@@ -14488,10 +14488,10 @@
         <v>46271</v>
       </c>
       <c r="B525" t="n">
-        <v>715.7</v>
+        <v>570.2</v>
       </c>
       <c r="C525" t="n">
-        <v>301.0859600036784</v>
+        <v>155.5859600036785</v>
       </c>
       <c r="D525" t="n">
         <v>876</v>
@@ -14500,10 +14500,10 @@
         <v>-414.6140399963223</v>
       </c>
       <c r="F525" t="n">
-        <v>-86.00000000000011</v>
+        <v>-231.5000000000001</v>
       </c>
       <c r="G525" t="n">
-        <v>-282.9588570093455</v>
+        <v>-428.4588570093455</v>
       </c>
       <c r="H525" t="n">
         <v>-309</v>
@@ -14514,10 +14514,10 @@
         <v>46272</v>
       </c>
       <c r="B526" t="n">
-        <v>715.7</v>
+        <v>570.2</v>
       </c>
       <c r="C526" t="n">
-        <v>301.0859600036784</v>
+        <v>155.5859600036785</v>
       </c>
       <c r="D526" t="n">
         <v>876</v>
@@ -14526,10 +14526,10 @@
         <v>-414.6140399963223</v>
       </c>
       <c r="F526" t="n">
-        <v>-86.00000000000011</v>
+        <v>-231.5000000000001</v>
       </c>
       <c r="G526" t="n">
-        <v>-282.9588570093455</v>
+        <v>-428.4588570093455</v>
       </c>
       <c r="H526" t="n">
         <v>-309</v>
@@ -14540,10 +14540,10 @@
         <v>46273</v>
       </c>
       <c r="B527" t="n">
-        <v>780.1</v>
+        <v>634.6</v>
       </c>
       <c r="C527" t="n">
-        <v>361.8059600036784</v>
+        <v>216.3059600036785</v>
       </c>
       <c r="D527" t="n">
         <v>930</v>
@@ -14552,10 +14552,10 @@
         <v>-418.2940399963223</v>
       </c>
       <c r="F527" t="n">
-        <v>-21.60000000000014</v>
+        <v>-167.1000000000001</v>
       </c>
       <c r="G527" t="n">
-        <v>-222.2388570093455</v>
+        <v>-367.7388570093455</v>
       </c>
       <c r="H527" t="n">
         <v>-255</v>
@@ -14566,10 +14566,10 @@
         <v>46274</v>
       </c>
       <c r="B528" t="n">
-        <v>780.1</v>
+        <v>634.6</v>
       </c>
       <c r="C528" t="n">
-        <v>356.6659600036784</v>
+        <v>211.1659600036785</v>
       </c>
       <c r="D528" t="n">
         <v>930</v>
@@ -14578,10 +14578,10 @@
         <v>-423.4340399963223</v>
       </c>
       <c r="F528" t="n">
-        <v>-21.60000000000014</v>
+        <v>-167.1000000000001</v>
       </c>
       <c r="G528" t="n">
-        <v>-227.3788570093455</v>
+        <v>-372.8788570093454</v>
       </c>
       <c r="H528" t="n">
         <v>-255</v>
@@ -14592,10 +14592,10 @@
         <v>46275</v>
       </c>
       <c r="B529" t="n">
-        <v>780.1</v>
+        <v>634.6</v>
       </c>
       <c r="C529" t="n">
-        <v>352.9659600036784</v>
+        <v>207.4659600036785</v>
       </c>
       <c r="D529" t="n">
         <v>930</v>
@@ -14604,10 +14604,10 @@
         <v>-427.1340399963223</v>
       </c>
       <c r="F529" t="n">
-        <v>-21.60000000000014</v>
+        <v>-167.1000000000001</v>
       </c>
       <c r="G529" t="n">
-        <v>-231.0788570093455</v>
+        <v>-376.5788570093454</v>
       </c>
       <c r="H529" t="n">
         <v>-255</v>
@@ -14618,10 +14618,10 @@
         <v>46276</v>
       </c>
       <c r="B530" t="n">
-        <v>780.1</v>
+        <v>634.6</v>
       </c>
       <c r="C530" t="n">
-        <v>348.6659600036784</v>
+        <v>203.1659600036785</v>
       </c>
       <c r="D530" t="n">
         <v>930</v>
@@ -14630,10 +14630,10 @@
         <v>-431.4340399963223</v>
       </c>
       <c r="F530" t="n">
-        <v>-21.60000000000014</v>
+        <v>-167.1000000000001</v>
       </c>
       <c r="G530" t="n">
-        <v>-235.3788570093455</v>
+        <v>-380.8788570093454</v>
       </c>
       <c r="H530" t="n">
         <v>-255</v>
@@ -14644,10 +14644,10 @@
         <v>46277</v>
       </c>
       <c r="B531" t="n">
-        <v>780.1</v>
+        <v>634.6</v>
       </c>
       <c r="C531" t="n">
-        <v>348.6659600036784</v>
+        <v>203.1659600036785</v>
       </c>
       <c r="D531" t="n">
         <v>930</v>
@@ -14656,10 +14656,10 @@
         <v>-431.4340399963223</v>
       </c>
       <c r="F531" t="n">
-        <v>-21.60000000000014</v>
+        <v>-167.1000000000001</v>
       </c>
       <c r="G531" t="n">
-        <v>-235.3788570093455</v>
+        <v>-380.8788570093454</v>
       </c>
       <c r="H531" t="n">
         <v>-255</v>
@@ -14670,10 +14670,10 @@
         <v>46278</v>
       </c>
       <c r="B532" t="n">
-        <v>780.1</v>
+        <v>634.6</v>
       </c>
       <c r="C532" t="n">
-        <v>348.6659600036784</v>
+        <v>203.1659600036785</v>
       </c>
       <c r="D532" t="n">
         <v>930</v>
@@ -14682,10 +14682,10 @@
         <v>-431.4340399963223</v>
       </c>
       <c r="F532" t="n">
-        <v>-21.60000000000014</v>
+        <v>-167.1000000000001</v>
       </c>
       <c r="G532" t="n">
-        <v>-235.3788570093455</v>
+        <v>-380.8788570093454</v>
       </c>
       <c r="H532" t="n">
         <v>-255</v>
@@ -14696,10 +14696,10 @@
         <v>46279</v>
       </c>
       <c r="B533" t="n">
-        <v>780.1</v>
+        <v>634.6</v>
       </c>
       <c r="C533" t="n">
-        <v>348.6659600036784</v>
+        <v>203.1659600036785</v>
       </c>
       <c r="D533" t="n">
         <v>930</v>
@@ -14708,10 +14708,10 @@
         <v>-431.4340399963223</v>
       </c>
       <c r="F533" t="n">
-        <v>-21.60000000000014</v>
+        <v>-167.1000000000001</v>
       </c>
       <c r="G533" t="n">
-        <v>-235.3788570093455</v>
+        <v>-380.8788570093454</v>
       </c>
       <c r="H533" t="n">
         <v>-255</v>
@@ -14722,10 +14722,10 @@
         <v>46280</v>
       </c>
       <c r="B534" t="n">
-        <v>948.7</v>
+        <v>803.2</v>
       </c>
       <c r="C534" t="n">
-        <v>510.6459600036784</v>
+        <v>365.1459600036785</v>
       </c>
       <c r="D534" t="n">
         <v>1105</v>
@@ -14737,7 +14737,7 @@
         <v>0</v>
       </c>
       <c r="G534" t="n">
-        <v>-73.39885700934553</v>
+        <v>-218.8988570093454</v>
       </c>
       <c r="H534" t="n">
         <v>-80</v>
@@ -14748,10 +14748,10 @@
         <v>46281</v>
       </c>
       <c r="B535" t="n">
-        <v>948.7</v>
+        <v>803.2</v>
       </c>
       <c r="C535" t="n">
-        <v>518.7459600036784</v>
+        <v>373.2459600036785</v>
       </c>
       <c r="D535" t="n">
         <v>1105</v>
@@ -14763,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="G535" t="n">
-        <v>-65.29885700934551</v>
+        <v>-210.7988570093454</v>
       </c>
       <c r="H535" t="n">
         <v>-80</v>
@@ -14774,10 +14774,10 @@
         <v>46282</v>
       </c>
       <c r="B536" t="n">
-        <v>948.7</v>
+        <v>803.2</v>
       </c>
       <c r="C536" t="n">
-        <v>512.3459600036784</v>
+        <v>366.8459600036786</v>
       </c>
       <c r="D536" t="n">
         <v>1105</v>
@@ -14789,7 +14789,7 @@
         <v>0</v>
       </c>
       <c r="G536" t="n">
-        <v>-71.69885700934549</v>
+        <v>-217.1988570093454</v>
       </c>
       <c r="H536" t="n">
         <v>-80</v>
@@ -14800,10 +14800,10 @@
         <v>46283</v>
       </c>
       <c r="B537" t="n">
-        <v>985.2</v>
+        <v>839.7</v>
       </c>
       <c r="C537" t="n">
-        <v>547.1459600036784</v>
+        <v>401.6459600036786</v>
       </c>
       <c r="D537" t="n">
         <v>1142</v>
@@ -14815,7 +14815,7 @@
         <v>0</v>
       </c>
       <c r="G537" t="n">
-        <v>-36.89885700934553</v>
+        <v>-182.3988570093454</v>
       </c>
       <c r="H537" t="n">
         <v>-43</v>
@@ -14826,10 +14826,10 @@
         <v>46284</v>
       </c>
       <c r="B538" t="n">
-        <v>985.2</v>
+        <v>839.7</v>
       </c>
       <c r="C538" t="n">
-        <v>547.1459600036784</v>
+        <v>401.6459600036786</v>
       </c>
       <c r="D538" t="n">
         <v>1142</v>
@@ -14841,7 +14841,7 @@
         <v>0</v>
       </c>
       <c r="G538" t="n">
-        <v>-36.89885700934553</v>
+        <v>-182.3988570093454</v>
       </c>
       <c r="H538" t="n">
         <v>-43</v>
@@ -14852,10 +14852,10 @@
         <v>46285</v>
       </c>
       <c r="B539" t="n">
-        <v>985.2</v>
+        <v>839.7</v>
       </c>
       <c r="C539" t="n">
-        <v>547.1459600036784</v>
+        <v>401.6459600036786</v>
       </c>
       <c r="D539" t="n">
         <v>1142</v>
@@ -14867,7 +14867,7 @@
         <v>0</v>
       </c>
       <c r="G539" t="n">
-        <v>-36.89885700934553</v>
+        <v>-182.3988570093454</v>
       </c>
       <c r="H539" t="n">
         <v>-43</v>
@@ -14878,10 +14878,10 @@
         <v>46286</v>
       </c>
       <c r="B540" t="n">
-        <v>993.8000000000001</v>
+        <v>848.3000000000001</v>
       </c>
       <c r="C540" t="n">
-        <v>553.2459600036784</v>
+        <v>407.7459600036786</v>
       </c>
       <c r="D540" t="n">
         <v>1154</v>
@@ -14893,7 +14893,7 @@
         <v>0</v>
       </c>
       <c r="G540" t="n">
-        <v>-30.79885700934551</v>
+        <v>-176.2988570093453</v>
       </c>
       <c r="H540" t="n">
         <v>-31</v>
@@ -14904,10 +14904,10 @@
         <v>46287</v>
       </c>
       <c r="B541" t="n">
-        <v>996.4000000000001</v>
+        <v>850.9000000000001</v>
       </c>
       <c r="C541" t="n">
-        <v>551.6059600036784</v>
+        <v>406.1059600036786</v>
       </c>
       <c r="D541" t="n">
         <v>1152</v>
@@ -14919,7 +14919,7 @@
         <v>0</v>
       </c>
       <c r="G541" t="n">
-        <v>-32.4388570093455</v>
+        <v>-177.9388570093453</v>
       </c>
       <c r="H541" t="n">
         <v>-33</v>
@@ -14930,10 +14930,10 @@
         <v>46288</v>
       </c>
       <c r="B542" t="n">
-        <v>998.2</v>
+        <v>852.7</v>
       </c>
       <c r="C542" t="n">
-        <v>550.0059600036784</v>
+        <v>404.5059600036786</v>
       </c>
       <c r="D542" t="n">
         <v>1152</v>
@@ -14945,7 +14945,7 @@
         <v>0</v>
       </c>
       <c r="G542" t="n">
-        <v>-34.03885700934552</v>
+        <v>-179.5388570093453</v>
       </c>
       <c r="H542" t="n">
         <v>-33</v>
@@ -14956,10 +14956,10 @@
         <v>46289</v>
       </c>
       <c r="B543" t="n">
-        <v>889</v>
+        <v>743.5</v>
       </c>
       <c r="C543" t="n">
-        <v>440.8059600036784</v>
+        <v>295.3059600036786</v>
       </c>
       <c r="D543" t="n">
         <v>1049</v>
@@ -14971,7 +14971,7 @@
         <v>-109.2</v>
       </c>
       <c r="G543" t="n">
-        <v>-143.2388570093455</v>
+        <v>-288.7388570093453</v>
       </c>
       <c r="H543" t="n">
         <v>-136</v>
@@ -14982,10 +14982,10 @@
         <v>46290</v>
       </c>
       <c r="B544" t="n">
-        <v>889</v>
+        <v>743.5</v>
       </c>
       <c r="C544" t="n">
-        <v>435.3100721532111</v>
+        <v>289.8100721532113</v>
       </c>
       <c r="D544" t="n">
         <v>1088</v>
@@ -14997,7 +14997,7 @@
         <v>-109.2</v>
       </c>
       <c r="G544" t="n">
-        <v>-148.7347448598128</v>
+        <v>-294.2347448598126</v>
       </c>
       <c r="H544" t="n">
         <v>-97</v>
@@ -15008,10 +15008,10 @@
         <v>46291</v>
       </c>
       <c r="B545" t="n">
-        <v>889</v>
+        <v>743.5</v>
       </c>
       <c r="C545" t="n">
-        <v>435.3100721532111</v>
+        <v>289.8100721532113</v>
       </c>
       <c r="D545" t="n">
         <v>1088</v>
@@ -15023,7 +15023,7 @@
         <v>-109.2</v>
       </c>
       <c r="G545" t="n">
-        <v>-148.7347448598128</v>
+        <v>-294.2347448598126</v>
       </c>
       <c r="H545" t="n">
         <v>-97</v>
@@ -15034,10 +15034,10 @@
         <v>46292</v>
       </c>
       <c r="B546" t="n">
-        <v>889</v>
+        <v>743.5</v>
       </c>
       <c r="C546" t="n">
-        <v>435.3100721532111</v>
+        <v>289.8100721532113</v>
       </c>
       <c r="D546" t="n">
         <v>1088</v>
@@ -15049,7 +15049,7 @@
         <v>-109.2</v>
       </c>
       <c r="G546" t="n">
-        <v>-148.7347448598128</v>
+        <v>-294.2347448598126</v>
       </c>
       <c r="H546" t="n">
         <v>-97</v>
@@ -15060,10 +15060,10 @@
         <v>46293</v>
       </c>
       <c r="B547" t="n">
-        <v>1010.8</v>
+        <v>865.3</v>
       </c>
       <c r="C547" t="n">
-        <v>553.4913805644261</v>
+        <v>407.9913805644263</v>
       </c>
       <c r="D547" t="n">
         <v>1088</v>
@@ -15075,7 +15075,7 @@
         <v>0</v>
       </c>
       <c r="G547" t="n">
-        <v>-30.55343644859784</v>
+        <v>-176.0534364485977</v>
       </c>
       <c r="H547" t="n">
         <v>-97</v>
@@ -15086,10 +15086,10 @@
         <v>46294</v>
       </c>
       <c r="B548" t="n">
-        <v>1043.8</v>
+        <v>898.3</v>
       </c>
       <c r="C548" t="n">
-        <v>579.3670814990055</v>
+        <v>433.8670814990057</v>
       </c>
       <c r="D548" t="n">
         <v>1088</v>
@@ -15101,7 +15101,7 @@
         <v>0</v>
       </c>
       <c r="G548" t="n">
-        <v>-4.677735514018423</v>
+        <v>-150.1777355140183</v>
       </c>
       <c r="H548" t="n">
         <v>-97</v>
@@ -15112,10 +15112,10 @@
         <v>46295</v>
       </c>
       <c r="B549" t="n">
-        <v>1043.8</v>
+        <v>898.3</v>
       </c>
       <c r="C549" t="n">
-        <v>576.5207263588186</v>
+        <v>431.0207263588188</v>
       </c>
       <c r="D549" t="n">
         <v>1088</v>
@@ -15127,7 +15127,7 @@
         <v>0</v>
       </c>
       <c r="G549" t="n">
-        <v>-7.524090654205338</v>
+        <v>-153.0240906542052</v>
       </c>
       <c r="H549" t="n">
         <v>-97</v>
@@ -15144,7 +15144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15180,7 +15180,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>live: exit date missing (open trade, -39.5 pts as logged; SSR exit was -185) (row 214): Exit NaT -&gt; 2026-04-30</t>
+          <t>live: exit date missing (open trade, closed at SSR exit) (row 214): Exit NaT -&gt; 2026-04-30</t>
         </is>
       </c>
     </row>
@@ -15190,7 +15190,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>live: year/month typo (row 277): Entry 2026-09-23 00:00:00 -&gt; 2026-09-23</t>
+          <t>live (row 214): open 24300 PE trade closed at model exit 388, net -39.5 -&gt; -185.0 pts (confirmed)</t>
         </is>
       </c>
     </row>
@@ -15200,7 +15200,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>live: month typo (row 277): Exit 2026-08-24 00:00:00 -&gt; 2026-09-24</t>
+          <t>live: year/month typo (row 277): Entry 2026-09-23 00:00:00 -&gt; 2026-09-23</t>
         </is>
       </c>
     </row>
@@ -15210,7 +15210,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>live: month typo (row 278): Entry 2026-08-24 00:00:00 -&gt; 2026-09-24</t>
+          <t>live: month typo (row 277): Exit 2026-08-24 00:00:00 -&gt; 2026-09-24</t>
         </is>
       </c>
     </row>
@@ -15220,7 +15220,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>hedge: exit typo (row 13): Exit 2025-06-27 00:00:00 -&gt; 2025-05-27</t>
+          <t>live: month typo (row 278): Entry 2026-08-24 00:00:00 -&gt; 2026-09-24</t>
         </is>
       </c>
     </row>
@@ -15230,7 +15230,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>hedge: entry year typo (row 114): Entry 2025-01-01 00:00:00 -&gt; 2026-01-01</t>
+          <t>hedge: exit typo (row 13): Exit 2025-06-27 00:00:00 -&gt; 2025-05-27</t>
         </is>
       </c>
     </row>
@@ -15240,7 +15240,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>hedge: exit month typo (the +221pt Budget-week hedge win) (row 133): Exit 2026-03-03 00:00:00 -&gt; 2026-02-03</t>
+          <t>hedge: entry year typo (row 114): Entry 2025-01-01 00:00:00 -&gt; 2026-01-01</t>
         </is>
       </c>
     </row>
@@ -15250,7 +15250,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>hedge: month typo (row 240): Exit 2026-08-02 00:00:00 -&gt; 2026-09-02</t>
+          <t>hedge: exit month typo (the +221pt Budget-week hedge win) (row 133): Exit 2026-03-03 00:00:00 -&gt; 2026-02-03</t>
         </is>
       </c>
     </row>
@@ -15259,6 +15259,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="inlineStr">
+        <is>
+          <t>hedge: month typo (row 240): Exit 2026-08-02 00:00:00 -&gt; 2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>hedge: month typo (row 241): Entry 2026-08-02 00:00:00 -&gt; 2026-09-02</t>
         </is>
@@ -15320,13 +15330,13 @@
         <v>45783</v>
       </c>
       <c r="C2" t="n">
-        <v>1084.2</v>
+        <v>938.7</v>
       </c>
       <c r="D2" t="n">
         <v>-1422.3</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7622864374604513</v>
+        <v>0.6599873444421007</v>
       </c>
       <c r="F2" t="n">
         <v>-797.8</v>
@@ -15342,13 +15352,13 @@
         <v>45783</v>
       </c>
       <c r="C3" t="n">
-        <v>616.9207263588185</v>
+        <v>471.4207263588184</v>
       </c>
       <c r="D3" t="n">
         <v>-1154.59</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5343201711073355</v>
+        <v>0.4083014112012216</v>
       </c>
       <c r="F3" t="n">
         <v>-576.48</v>
@@ -15474,7 +15484,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1426.6</v>
+        <v>1281.1</v>
       </c>
     </row>
     <row r="10">
@@ -15494,7 +15504,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-164.3999999999999</v>
+        <v>-309.8999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -15504,7 +15514,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.6347490347490342</v>
+        <v>-1.196525096525096</v>
       </c>
     </row>
     <row r="13">
@@ -15524,7 +15534,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>14.679327770486</v>
+        <v>11.50628861973853</v>
       </c>
     </row>
     <row r="15">
@@ -15544,7 +15554,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>69.1119691119691</v>
+        <v>69.4980694980695</v>
       </c>
     </row>
     <row r="17">
@@ -15554,7 +15564,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.9897276818665749</v>
+        <v>0.9937501116066584</v>
       </c>
     </row>
     <row r="18">
@@ -15564,7 +15574,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1043.8</v>
+        <v>898.3</v>
       </c>
     </row>
     <row r="19">
@@ -15584,7 +15594,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-44.20000000000027</v>
+        <v>-189.7</v>
       </c>
     </row>
     <row r="21">
@@ -15594,7 +15604,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-164.3999999999999</v>
+        <v>-309.8999999999999</v>
       </c>
     </row>
     <row r="22">
@@ -16115,19 +16125,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>320.7</v>
+        <v>175.2</v>
       </c>
       <c r="C14" t="n">
         <v>-261.2</v>
       </c>
       <c r="D14" t="n">
-        <v>59.5</v>
+        <v>-86</v>
       </c>
       <c r="E14" t="n">
         <v>115</v>
       </c>
       <c r="F14" t="n">
-        <v>205.7</v>
+        <v>60.2</v>
       </c>
     </row>
     <row r="15">
@@ -24479,13 +24489,13 @@
         <v>203</v>
       </c>
       <c r="J191" t="n">
-        <v>-39.5</v>
+        <v>-185</v>
       </c>
       <c r="K191" t="n">
         <v>-185</v>
       </c>
       <c r="L191" t="n">
-        <v>145.5</v>
+        <v>0</v>
       </c>
       <c r="M191" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Add hedged result (-475) for Apr 30-May 24 2026 missed trades to analysis and report
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NXDNZiScC3GTCLADanc7h1
</commit_message>
<xml_diff>
--- a/analysis/ssr_live_vs_model_analysis.xlsx
+++ b/analysis/ssr_live_vs_model_analysis.xlsx
@@ -15638,7 +15638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15657,6 +15657,16 @@
           <t>model pts not captured</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>model pts incl. hedge (supplied)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>hedge effect (pts)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -15670,6 +15680,12 @@
       <c r="C2" t="n">
         <v>-553</v>
       </c>
+      <c r="D2" t="n">
+        <v>-475</v>
+      </c>
+      <c r="E2" t="n">
+        <v>78</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -15683,6 +15699,8 @@
       <c r="C3" t="n">
         <v>155</v>
       </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -15696,6 +15714,8 @@
       <c r="C4" t="n">
         <v>370</v>
       </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -15709,6 +15729,8 @@
       <c r="C5" t="n">
         <v>-475</v>
       </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>